<commit_message>
Actualizar inventario (1 cambios)
</commit_message>
<xml_diff>
--- a/inventario.xlsx
+++ b/inventario.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="27932"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{26F1DF04-64D2-4F9C-BE26-8B8C4B1D96B5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6F40A863-FBA8-4B35-8393-DBDDA70BB5D8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="20370" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -378,7 +378,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="&quot;$&quot;\ #,##0"/>
   </numFmts>
-  <fonts count="13" x14ac:knownFonts="1">
+  <fonts count="14" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -450,6 +450,12 @@
       <color rgb="FF2E8B80"/>
       <name val="Arial"/>
     </font>
+    <font>
+      <u/>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="7">
     <fill>
@@ -496,7 +502,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -550,6 +556,9 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -933,7 +942,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:H32"/>
+  <dimension ref="A1:L32"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="52" customWidth="1"/>
@@ -945,7 +954,7 @@
     <col min="7" max="8" width="20" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:12" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="18" t="s">
         <v>0</v>
       </c>
@@ -956,7 +965,7 @@
       <c r="F1" s="18"/>
       <c r="G1" s="18"/>
     </row>
-    <row r="2" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:12" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="19" t="s">
         <v>1</v>
       </c>
@@ -967,7 +976,7 @@
       <c r="F2" s="19"/>
       <c r="G2" s="19"/>
     </row>
-    <row r="4" spans="1:8" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:12" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
         <v>2</v>
       </c>
@@ -993,7 +1002,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="5" spans="1:8" s="2" customFormat="1" ht="12.75" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:12" s="2" customFormat="1" ht="12.75" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
         <v>10</v>
       </c>
@@ -1020,7 +1029,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="6" spans="1:8" s="2" customFormat="1" ht="12.75" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:12" s="2" customFormat="1" ht="12.75" x14ac:dyDescent="0.25">
       <c r="A6" s="10" t="s">
         <v>15</v>
       </c>
@@ -1047,7 +1056,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="7" spans="1:8" s="2" customFormat="1" ht="12.75" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:12" s="2" customFormat="1" ht="12.75" x14ac:dyDescent="0.25">
       <c r="A7" s="3" t="s">
         <v>18</v>
       </c>
@@ -1074,7 +1083,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="8" spans="1:8" s="2" customFormat="1" ht="12.75" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:12" s="2" customFormat="1" ht="12.75" x14ac:dyDescent="0.25">
       <c r="A8" s="10" t="s">
         <v>21</v>
       </c>
@@ -1101,7 +1110,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="9" spans="1:8" s="2" customFormat="1" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:12" s="2" customFormat="1" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A9" s="3" t="s">
         <v>24</v>
       </c>
@@ -1128,7 +1137,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="10" spans="1:8" s="2" customFormat="1" ht="12.75" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:12" s="2" customFormat="1" ht="12.75" x14ac:dyDescent="0.25">
       <c r="A10" s="10" t="s">
         <v>26</v>
       </c>
@@ -1155,7 +1164,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="11" spans="1:8" s="2" customFormat="1" ht="12.75" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:12" s="2" customFormat="1" ht="12.75" x14ac:dyDescent="0.25">
       <c r="A11" s="3" t="s">
         <v>28</v>
       </c>
@@ -1182,7 +1191,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="12" spans="1:8" s="2" customFormat="1" ht="12.75" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:12" s="2" customFormat="1" ht="12.75" x14ac:dyDescent="0.25">
       <c r="A12" s="10" t="s">
         <v>30</v>
       </c>
@@ -1209,7 +1218,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="13" spans="1:8" s="2" customFormat="1" ht="12.75" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:12" s="2" customFormat="1" ht="12.75" x14ac:dyDescent="0.25">
       <c r="A13" s="3" t="s">
         <v>34</v>
       </c>
@@ -1223,20 +1232,20 @@
         <v>160000</v>
       </c>
       <c r="E13" s="6">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F13" s="7" t="s">
         <v>13</v>
       </c>
       <c r="G13" s="8" t="str">
         <f t="shared" si="0"/>
-        <v>Últimas unidades</v>
+        <v>AGOTADO</v>
       </c>
       <c r="H13" s="9" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="14" spans="1:8" s="2" customFormat="1" ht="12.75" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:12" s="2" customFormat="1" ht="12.75" x14ac:dyDescent="0.25">
       <c r="A14" s="10" t="s">
         <v>36</v>
       </c>
@@ -1263,7 +1272,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="15" spans="1:8" s="2" customFormat="1" ht="12.75" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:12" s="2" customFormat="1" ht="12.75" x14ac:dyDescent="0.25">
       <c r="A15" s="3" t="s">
         <v>38</v>
       </c>
@@ -1290,7 +1299,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="16" spans="1:8" s="2" customFormat="1" ht="12.75" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:12" s="2" customFormat="1" ht="12.75" x14ac:dyDescent="0.25">
       <c r="A16" s="10" t="s">
         <v>40</v>
       </c>
@@ -1316,6 +1325,7 @@
       <c r="H16" s="9" t="s">
         <v>41</v>
       </c>
+      <c r="L16" s="21"/>
     </row>
     <row r="17" spans="1:8" s="2" customFormat="1" ht="12.75" x14ac:dyDescent="0.25">
       <c r="A17" s="3" t="s">
@@ -1868,7 +1878,7 @@
       </c>
       <c r="B5" s="12">
         <f>COUNTIF(Inventario!$G$5:$G$32,"Últimas unidades")</f>
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
@@ -1877,7 +1887,7 @@
       </c>
       <c r="B6" s="12">
         <f>COUNTIF(Inventario!$G$5:$G$32,"AGOTADO")</f>
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
@@ -1895,7 +1905,7 @@
       </c>
       <c r="B8" s="12">
         <f>SUM(Inventario!$E$5:$E$32)</f>
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
@@ -1904,7 +1914,7 @@
       </c>
       <c r="B9" s="13">
         <f>SUMPRODUCT(Inventario!$D$5:$D$32,Inventario!$E$5:$E$32)</f>
-        <v>4870000</v>
+        <v>4710000</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Actualizar inventario (2 cambios)
</commit_message>
<xml_diff>
--- a/inventario.xlsx
+++ b/inventario.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="27932"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6F40A863-FBA8-4B35-8393-DBDDA70BB5D8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2EC93B7E-7496-4223-AD90-4AF2E937945A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="20370" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -549,6 +549,9 @@
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -556,9 +559,6 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -955,26 +955,26 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:12" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="18" t="s">
+      <c r="A1" s="19" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="18"/>
-      <c r="C1" s="18"/>
-      <c r="D1" s="18"/>
-      <c r="E1" s="18"/>
-      <c r="F1" s="18"/>
-      <c r="G1" s="18"/>
+      <c r="B1" s="19"/>
+      <c r="C1" s="19"/>
+      <c r="D1" s="19"/>
+      <c r="E1" s="19"/>
+      <c r="F1" s="19"/>
+      <c r="G1" s="19"/>
     </row>
     <row r="2" spans="1:12" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="19" t="s">
+      <c r="A2" s="20" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="19"/>
-      <c r="C2" s="19"/>
-      <c r="D2" s="19"/>
-      <c r="E2" s="19"/>
-      <c r="F2" s="19"/>
-      <c r="G2" s="19"/>
+      <c r="B2" s="20"/>
+      <c r="C2" s="20"/>
+      <c r="D2" s="20"/>
+      <c r="E2" s="20"/>
+      <c r="F2" s="20"/>
+      <c r="G2" s="20"/>
     </row>
     <row r="4" spans="1:12" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
@@ -1043,7 +1043,7 @@
         <v>130000</v>
       </c>
       <c r="E6" s="6">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F6" s="7" t="s">
         <v>13</v>
@@ -1151,7 +1151,7 @@
         <v>130000</v>
       </c>
       <c r="E10" s="6">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F10" s="7" t="s">
         <v>13</v>
@@ -1325,7 +1325,7 @@
       <c r="H16" s="9" t="s">
         <v>41</v>
       </c>
-      <c r="L16" s="21"/>
+      <c r="L16" s="18"/>
     </row>
     <row r="17" spans="1:8" s="2" customFormat="1" ht="12.75" x14ac:dyDescent="0.25">
       <c r="A17" s="3" t="s">
@@ -1849,10 +1849,10 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:2" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="20" t="s">
+      <c r="A1" s="21" t="s">
         <v>80</v>
       </c>
-      <c r="B1" s="20"/>
+      <c r="B1" s="21"/>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" s="11" t="s">
@@ -1905,7 +1905,7 @@
       </c>
       <c r="B8" s="12">
         <f>SUM(Inventario!$E$5:$E$32)</f>
-        <v>40</v>
+        <v>38</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
@@ -1914,7 +1914,7 @@
       </c>
       <c r="B9" s="13">
         <f>SUMPRODUCT(Inventario!$D$5:$D$32,Inventario!$E$5:$E$32)</f>
-        <v>4710000</v>
+        <v>4450000</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Agregar CoQ10 200mg Nature Made (#29), $260.000, stock 1
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/inventario.xlsx
+++ b/inventario.xlsx
@@ -1,39 +1,19 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="27932"/>
-  <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2EC93B7E-7496-4223-AD90-4AF2E937945A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
-  <bookViews>
-    <workbookView xWindow="20370" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
-  </bookViews>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
+  <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
   <sheets>
-    <sheet name="Inventario" sheetId="1" r:id="rId1"/>
-    <sheet name="Resumen" sheetId="2" r:id="rId2"/>
-    <sheet name="Instrucciones" sheetId="3" r:id="rId3"/>
+    <sheet sheetId="1" name="Inventario" state="visible" r:id="rId4"/>
+    <sheet sheetId="2" name="Resumen" state="visible" r:id="rId5"/>
+    <sheet sheetId="3" name="Instrucciones" state="visible" r:id="rId6"/>
   </sheets>
-  <calcPr calcId="191029"/>
-  <extLst>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
-    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
-      <xlwcv:version setVersion="1"/>
-    </ext>
-  </extLst>
+  <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="185" uniqueCount="112">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="190" uniqueCount="114">
   <si>
     <t>INVENTARIO — El Garaje de Rochi</t>
   </si>
@@ -275,6 +255,12 @@
     <t>SUP-GLUCO-280</t>
   </si>
   <si>
+    <t>Nature Made CoQ10 200 mg (140 softgels)</t>
+  </si>
+  <si>
+    <t>SUP-COQ10-140</t>
+  </si>
+  <si>
     <t>RESUMEN DEL INVENTARIO</t>
   </si>
   <si>
@@ -302,7 +288,7 @@
     <t>Se recalcula solo cuando cambias las cantidades en la hoja Inventario.</t>
   </si>
   <si>
-    <t>Generado: 1/9/2026, 8:37:30 p. m.</t>
+    <t>Generado: 25/9/2026, 10:55:35 a. m.</t>
   </si>
   <si>
     <t>CÓMO USAR ESTE EXCEL</t>
@@ -374,34 +360,34 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="&quot;$&quot;\ #,##0"/>
+    <numFmt numFmtId="164" formatCode="&quot;$&quot; #,##0"/>
   </numFmts>
-  <fonts count="14" x14ac:knownFonts="1">
+  <fonts count="13" x14ac:knownFonts="1">
     <font>
-      <sz val="11"/>
       <color theme="1"/>
-      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+      <sz val="11"/>
+      <name val="Calibri"/>
     </font>
     <font>
       <b/>
+      <color rgb="FFFFFFFF"/>
       <sz val="16"/>
-      <color rgb="FFFFFFFF"/>
       <name val="Arial"/>
     </font>
     <font>
       <i/>
+      <color rgb="FF6b7472"/>
       <sz val="9"/>
-      <color rgb="FF6B7472"/>
       <name val="Arial"/>
     </font>
     <font>
       <b/>
+      <color rgb="FFFFFFFF"/>
       <sz val="10"/>
-      <color rgb="FFFFFFFF"/>
       <name val="Arial"/>
     </font>
     <font>
@@ -414,14 +400,14 @@
       <name val="Arial"/>
     </font>
     <font>
+      <color rgb="FF9A9A9A"/>
       <sz val="8"/>
-      <color rgb="FF9A9A9A"/>
       <name val="Arial"/>
     </font>
     <font>
       <b/>
+      <color rgb="FFFFFFFF"/>
       <sz val="14"/>
-      <color rgb="FFFFFFFF"/>
       <name val="Arial"/>
     </font>
     <font>
@@ -434,27 +420,21 @@
       <name val="Arial"/>
     </font>
     <font>
+      <color rgb="FF9A9A9A"/>
       <sz val="9"/>
-      <color rgb="FF9A9A9A"/>
       <name val="Arial"/>
     </font>
     <font>
       <b/>
+      <color rgb="FFFFFFFF"/>
       <sz val="15"/>
-      <color rgb="FFFFFFFF"/>
       <name val="Arial"/>
     </font>
     <font>
       <b/>
+      <color rgb="FF2E8B80"/>
       <sz val="11"/>
-      <color rgb="FF2E8B80"/>
       <name val="Arial"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="10"/>
-      <name val="Arial"/>
-      <family val="2"/>
     </font>
   </fonts>
   <fills count="7">
@@ -502,8 +482,14 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -534,6 +520,7 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="1" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
@@ -549,16 +536,6 @@
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -566,21 +543,11 @@
   <dxfs count="4">
     <dxf>
       <font>
-        <color rgb="FF006100"/>
+        <color rgb="FF9C0006"/>
       </font>
       <fill>
         <patternFill patternType="solid">
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF6B7472"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFEDEDED"/>
+          <bgColor rgb="FFFFC7CE"/>
         </patternFill>
       </fill>
     </dxf>
@@ -596,11 +563,21 @@
     </dxf>
     <dxf>
       <font>
-        <color rgb="FF9C0006"/>
+        <color rgb="FF6b7472"/>
       </font>
       <fill>
         <patternFill patternType="solid">
-          <bgColor rgb="FFFFC7CE"/>
+          <bgColor rgb="FFEDEDED"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFC6EFCE"/>
         </patternFill>
       </fill>
     </dxf>
@@ -938,12 +915,12 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:L32"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:H33"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="52" customWidth="1"/>
     <col min="2" max="2" width="18" customWidth="1"/>
@@ -954,977 +931,920 @@
     <col min="7" max="8" width="20" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="19" t="s">
+    <row r="1" ht="28" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="19"/>
-      <c r="C1" s="19"/>
-      <c r="D1" s="19"/>
-      <c r="E1" s="19"/>
-      <c r="F1" s="19"/>
-      <c r="G1" s="19"/>
-    </row>
-    <row r="2" spans="1:12" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="20" t="s">
+      <c r="B1" s="1"/>
+      <c r="C1" s="1"/>
+      <c r="D1" s="1"/>
+      <c r="E1" s="1"/>
+      <c r="F1" s="1"/>
+      <c r="G1" s="1"/>
+    </row>
+    <row r="2" ht="30" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="20"/>
-      <c r="C2" s="20"/>
-      <c r="D2" s="20"/>
-      <c r="E2" s="20"/>
-      <c r="F2" s="20"/>
-      <c r="G2" s="20"/>
-    </row>
-    <row r="4" spans="1:12" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="1" t="s">
+      <c r="B2" s="2"/>
+      <c r="C2" s="2"/>
+      <c r="D2" s="2"/>
+      <c r="E2" s="2"/>
+      <c r="F2" s="2"/>
+      <c r="G2" s="2"/>
+    </row>
+    <row r="4" ht="32" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A4" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="1" t="s">
+      <c r="B4" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="C4" s="1" t="s">
+      <c r="C4" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="D4" s="1" t="s">
+      <c r="D4" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="E4" s="1" t="s">
+      <c r="E4" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="F4" s="1" t="s">
+      <c r="F4" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="G4" s="1" t="s">
+      <c r="G4" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="H4" s="1" t="s">
+      <c r="H4" s="3" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="5" spans="1:12" s="2" customFormat="1" ht="12.75" x14ac:dyDescent="0.25">
-      <c r="A5" s="3" t="s">
+    <row r="5" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="B5" s="4" t="s">
+      <c r="B5" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="C5" s="4" t="s">
+      <c r="C5" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="D5" s="5">
+      <c r="D5" s="7">
         <v>170000</v>
       </c>
-      <c r="E5" s="6">
+      <c r="E5" s="8">
         <v>2</v>
       </c>
-      <c r="F5" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="G5" s="8" t="str">
-        <f t="shared" ref="G5:G32" si="0">IF(F5="NO","Oculto",IF(E5&lt;=0,"AGOTADO",IF(E5&lt;=5,"Últimas unidades","Disponible")))</f>
-        <v>Últimas unidades</v>
-      </c>
-      <c r="H5" s="9" t="s">
+      <c r="F5" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="G5" s="10">
+        <f>IF(F5="NO","Oculto",IF(E5&lt;=0,"AGOTADO",IF(E5&lt;=5,"Últimas unidades","Disponible")))</f>
+      </c>
+      <c r="H5" s="11" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="6" spans="1:12" s="2" customFormat="1" ht="12.75" x14ac:dyDescent="0.25">
-      <c r="A6" s="10" t="s">
+    <row r="6" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="12" t="s">
         <v>15</v>
       </c>
-      <c r="B6" s="2" t="s">
+      <c r="B6" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="C6" s="2" t="s">
+      <c r="C6" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="D6" s="5">
+      <c r="D6" s="7">
         <v>130000</v>
       </c>
-      <c r="E6" s="6">
+      <c r="E6" s="8">
         <v>2</v>
       </c>
-      <c r="F6" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="G6" s="8" t="str">
-        <f t="shared" si="0"/>
-        <v>Últimas unidades</v>
-      </c>
-      <c r="H6" s="9" t="s">
+      <c r="F6" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="G6" s="10">
+        <f>IF(F6="NO","Oculto",IF(E6&lt;=0,"AGOTADO",IF(E6&lt;=5,"Últimas unidades","Disponible")))</f>
+      </c>
+      <c r="H6" s="11" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="7" spans="1:12" s="2" customFormat="1" ht="12.75" x14ac:dyDescent="0.25">
-      <c r="A7" s="3" t="s">
+    <row r="7" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="B7" s="4" t="s">
+      <c r="B7" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="C7" s="4" t="s">
+      <c r="C7" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="D7" s="5">
+      <c r="D7" s="7">
         <v>130000</v>
       </c>
-      <c r="E7" s="6">
+      <c r="E7" s="8">
         <v>1</v>
       </c>
-      <c r="F7" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="G7" s="8" t="str">
-        <f t="shared" si="0"/>
-        <v>Últimas unidades</v>
-      </c>
-      <c r="H7" s="9" t="s">
+      <c r="F7" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="G7" s="10">
+        <f>IF(F7="NO","Oculto",IF(E7&lt;=0,"AGOTADO",IF(E7&lt;=5,"Últimas unidades","Disponible")))</f>
+      </c>
+      <c r="H7" s="11" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="8" spans="1:12" s="2" customFormat="1" ht="12.75" x14ac:dyDescent="0.25">
-      <c r="A8" s="10" t="s">
+    <row r="8" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="12" t="s">
         <v>21</v>
       </c>
-      <c r="B8" s="2" t="s">
+      <c r="B8" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="C8" s="2" t="s">
+      <c r="C8" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="D8" s="5">
+      <c r="D8" s="7">
         <v>130000</v>
       </c>
-      <c r="E8" s="6">
+      <c r="E8" s="8">
         <v>1</v>
       </c>
-      <c r="F8" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="G8" s="8" t="str">
-        <f t="shared" si="0"/>
-        <v>Últimas unidades</v>
-      </c>
-      <c r="H8" s="9" t="s">
+      <c r="F8" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="G8" s="10">
+        <f>IF(F8="NO","Oculto",IF(E8&lt;=0,"AGOTADO",IF(E8&lt;=5,"Últimas unidades","Disponible")))</f>
+      </c>
+      <c r="H8" s="11" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="9" spans="1:12" s="2" customFormat="1" ht="25.5" x14ac:dyDescent="0.25">
-      <c r="A9" s="3" t="s">
+    <row r="9" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="5" t="s">
         <v>24</v>
       </c>
-      <c r="B9" s="4" t="s">
+      <c r="B9" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="C9" s="4" t="s">
+      <c r="C9" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="D9" s="5">
+      <c r="D9" s="7">
         <v>160000</v>
       </c>
-      <c r="E9" s="6">
+      <c r="E9" s="8">
         <v>0</v>
       </c>
-      <c r="F9" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="G9" s="8" t="str">
-        <f t="shared" si="0"/>
-        <v>AGOTADO</v>
-      </c>
-      <c r="H9" s="9" t="s">
+      <c r="F9" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="G9" s="10">
+        <f>IF(F9="NO","Oculto",IF(E9&lt;=0,"AGOTADO",IF(E9&lt;=5,"Últimas unidades","Disponible")))</f>
+      </c>
+      <c r="H9" s="11" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="10" spans="1:12" s="2" customFormat="1" ht="12.75" x14ac:dyDescent="0.25">
-      <c r="A10" s="10" t="s">
+    <row r="10" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="12" t="s">
         <v>26</v>
       </c>
-      <c r="B10" s="2" t="s">
+      <c r="B10" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="C10" s="2" t="s">
+      <c r="C10" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="D10" s="5">
+      <c r="D10" s="7">
         <v>130000</v>
       </c>
-      <c r="E10" s="6">
+      <c r="E10" s="8">
         <v>1</v>
       </c>
-      <c r="F10" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="G10" s="8" t="str">
-        <f t="shared" si="0"/>
-        <v>Últimas unidades</v>
-      </c>
-      <c r="H10" s="9" t="s">
+      <c r="F10" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="G10" s="10">
+        <f>IF(F10="NO","Oculto",IF(E10&lt;=0,"AGOTADO",IF(E10&lt;=5,"Últimas unidades","Disponible")))</f>
+      </c>
+      <c r="H10" s="11" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="11" spans="1:12" s="2" customFormat="1" ht="12.75" x14ac:dyDescent="0.25">
-      <c r="A11" s="3" t="s">
+    <row r="11" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="5" t="s">
         <v>28</v>
       </c>
-      <c r="B11" s="4" t="s">
+      <c r="B11" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="C11" s="4" t="s">
+      <c r="C11" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="D11" s="5">
+      <c r="D11" s="7">
         <v>120000</v>
       </c>
-      <c r="E11" s="6">
+      <c r="E11" s="8">
         <v>1</v>
       </c>
-      <c r="F11" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="G11" s="8" t="str">
-        <f t="shared" si="0"/>
-        <v>Últimas unidades</v>
-      </c>
-      <c r="H11" s="9" t="s">
+      <c r="F11" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="G11" s="10">
+        <f>IF(F11="NO","Oculto",IF(E11&lt;=0,"AGOTADO",IF(E11&lt;=5,"Últimas unidades","Disponible")))</f>
+      </c>
+      <c r="H11" s="11" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="12" spans="1:12" s="2" customFormat="1" ht="12.75" x14ac:dyDescent="0.25">
-      <c r="A12" s="10" t="s">
+    <row r="12" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="12" t="s">
         <v>30</v>
       </c>
-      <c r="B12" s="2" t="s">
+      <c r="B12" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="C12" s="2" t="s">
+      <c r="C12" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="D12" s="5">
+      <c r="D12" s="7">
         <v>160000</v>
       </c>
-      <c r="E12" s="6">
+      <c r="E12" s="8">
         <v>0</v>
       </c>
-      <c r="F12" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="G12" s="8" t="str">
-        <f t="shared" si="0"/>
-        <v>AGOTADO</v>
-      </c>
-      <c r="H12" s="9" t="s">
+      <c r="F12" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="G12" s="10">
+        <f>IF(F12="NO","Oculto",IF(E12&lt;=0,"AGOTADO",IF(E12&lt;=5,"Últimas unidades","Disponible")))</f>
+      </c>
+      <c r="H12" s="11" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="13" spans="1:12" s="2" customFormat="1" ht="12.75" x14ac:dyDescent="0.25">
-      <c r="A13" s="3" t="s">
+    <row r="13" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="5" t="s">
         <v>34</v>
       </c>
-      <c r="B13" s="4" t="s">
+      <c r="B13" s="6" t="s">
         <v>31</v>
       </c>
-      <c r="C13" s="4" t="s">
+      <c r="C13" s="6" t="s">
         <v>32</v>
       </c>
-      <c r="D13" s="5">
+      <c r="D13" s="7">
         <v>160000</v>
       </c>
-      <c r="E13" s="6">
+      <c r="E13" s="8">
         <v>0</v>
       </c>
-      <c r="F13" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="G13" s="8" t="str">
-        <f t="shared" si="0"/>
-        <v>AGOTADO</v>
-      </c>
-      <c r="H13" s="9" t="s">
+      <c r="F13" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="G13" s="10">
+        <f>IF(F13="NO","Oculto",IF(E13&lt;=0,"AGOTADO",IF(E13&lt;=5,"Últimas unidades","Disponible")))</f>
+      </c>
+      <c r="H13" s="11" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="14" spans="1:12" s="2" customFormat="1" ht="12.75" x14ac:dyDescent="0.25">
-      <c r="A14" s="10" t="s">
+    <row r="14" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="12" t="s">
         <v>36</v>
       </c>
-      <c r="B14" s="2" t="s">
+      <c r="B14" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="C14" s="2" t="s">
+      <c r="C14" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="D14" s="5">
+      <c r="D14" s="7">
         <v>160000</v>
       </c>
-      <c r="E14" s="6">
+      <c r="E14" s="8">
         <v>0</v>
       </c>
-      <c r="F14" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="G14" s="8" t="str">
-        <f t="shared" si="0"/>
-        <v>AGOTADO</v>
-      </c>
-      <c r="H14" s="9" t="s">
+      <c r="F14" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="G14" s="10">
+        <f>IF(F14="NO","Oculto",IF(E14&lt;=0,"AGOTADO",IF(E14&lt;=5,"Últimas unidades","Disponible")))</f>
+      </c>
+      <c r="H14" s="11" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="15" spans="1:12" s="2" customFormat="1" ht="12.75" x14ac:dyDescent="0.25">
-      <c r="A15" s="3" t="s">
+    <row r="15" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="5" t="s">
         <v>38</v>
       </c>
-      <c r="B15" s="4" t="s">
+      <c r="B15" s="6" t="s">
         <v>31</v>
       </c>
-      <c r="C15" s="4" t="s">
+      <c r="C15" s="6" t="s">
         <v>32</v>
       </c>
-      <c r="D15" s="5">
+      <c r="D15" s="7">
         <v>200000</v>
       </c>
-      <c r="E15" s="6">
+      <c r="E15" s="8">
         <v>0</v>
       </c>
-      <c r="F15" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="G15" s="8" t="str">
-        <f t="shared" si="0"/>
-        <v>AGOTADO</v>
-      </c>
-      <c r="H15" s="9" t="s">
+      <c r="F15" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="G15" s="10">
+        <f>IF(F15="NO","Oculto",IF(E15&lt;=0,"AGOTADO",IF(E15&lt;=5,"Últimas unidades","Disponible")))</f>
+      </c>
+      <c r="H15" s="11" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="16" spans="1:12" s="2" customFormat="1" ht="12.75" x14ac:dyDescent="0.25">
-      <c r="A16" s="10" t="s">
+    <row r="16" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="12" t="s">
         <v>40</v>
       </c>
-      <c r="B16" s="2" t="s">
+      <c r="B16" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="C16" s="2" t="s">
+      <c r="C16" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="D16" s="5">
+      <c r="D16" s="7">
         <v>130000</v>
       </c>
-      <c r="E16" s="6">
+      <c r="E16" s="8">
         <v>1</v>
       </c>
-      <c r="F16" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="G16" s="8" t="str">
-        <f t="shared" si="0"/>
-        <v>Últimas unidades</v>
-      </c>
-      <c r="H16" s="9" t="s">
+      <c r="F16" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="G16" s="10">
+        <f>IF(F16="NO","Oculto",IF(E16&lt;=0,"AGOTADO",IF(E16&lt;=5,"Últimas unidades","Disponible")))</f>
+      </c>
+      <c r="H16" s="11" t="s">
         <v>41</v>
       </c>
-      <c r="L16" s="18"/>
-    </row>
-    <row r="17" spans="1:8" s="2" customFormat="1" ht="12.75" x14ac:dyDescent="0.25">
-      <c r="A17" s="3" t="s">
+    </row>
+    <row r="17" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A17" s="5" t="s">
         <v>42</v>
       </c>
-      <c r="B17" s="4" t="s">
+      <c r="B17" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="C17" s="4" t="s">
+      <c r="C17" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="D17" s="5">
+      <c r="D17" s="7">
         <v>200000</v>
       </c>
-      <c r="E17" s="6">
+      <c r="E17" s="8">
         <v>1</v>
       </c>
-      <c r="F17" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="G17" s="8" t="str">
-        <f t="shared" si="0"/>
-        <v>Últimas unidades</v>
-      </c>
-      <c r="H17" s="9" t="s">
+      <c r="F17" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="G17" s="10">
+        <f>IF(F17="NO","Oculto",IF(E17&lt;=0,"AGOTADO",IF(E17&lt;=5,"Últimas unidades","Disponible")))</f>
+      </c>
+      <c r="H17" s="11" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="18" spans="1:8" s="2" customFormat="1" ht="25.5" x14ac:dyDescent="0.25">
-      <c r="A18" s="10" t="s">
+    <row r="18" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A18" s="12" t="s">
         <v>44</v>
       </c>
-      <c r="B18" s="2" t="s">
+      <c r="B18" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="C18" s="2" t="s">
+      <c r="C18" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="D18" s="5">
+      <c r="D18" s="7">
         <v>130000</v>
       </c>
-      <c r="E18" s="6">
+      <c r="E18" s="8">
         <v>0</v>
       </c>
-      <c r="F18" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="G18" s="8" t="str">
-        <f t="shared" si="0"/>
-        <v>AGOTADO</v>
-      </c>
-      <c r="H18" s="9" t="s">
+      <c r="F18" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="G18" s="10">
+        <f>IF(F18="NO","Oculto",IF(E18&lt;=0,"AGOTADO",IF(E18&lt;=5,"Últimas unidades","Disponible")))</f>
+      </c>
+      <c r="H18" s="11" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="19" spans="1:8" s="2" customFormat="1" ht="12.75" x14ac:dyDescent="0.25">
-      <c r="A19" s="3" t="s">
+    <row r="19" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="5" t="s">
         <v>46</v>
       </c>
-      <c r="B19" s="4" t="s">
+      <c r="B19" s="6" t="s">
         <v>22</v>
       </c>
-      <c r="C19" s="4" t="s">
+      <c r="C19" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="D19" s="5">
+      <c r="D19" s="7">
         <v>120000</v>
       </c>
-      <c r="E19" s="6">
+      <c r="E19" s="8">
         <v>4</v>
       </c>
-      <c r="F19" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="G19" s="8" t="str">
-        <f t="shared" si="0"/>
-        <v>Últimas unidades</v>
-      </c>
-      <c r="H19" s="9" t="s">
+      <c r="F19" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="G19" s="10">
+        <f>IF(F19="NO","Oculto",IF(E19&lt;=0,"AGOTADO",IF(E19&lt;=5,"Últimas unidades","Disponible")))</f>
+      </c>
+      <c r="H19" s="11" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="20" spans="1:8" s="2" customFormat="1" ht="12.75" x14ac:dyDescent="0.25">
-      <c r="A20" s="10" t="s">
+    <row r="20" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A20" s="12" t="s">
         <v>48</v>
       </c>
-      <c r="B20" s="2" t="s">
+      <c r="B20" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="C20" s="2" t="s">
+      <c r="C20" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="D20" s="5">
+      <c r="D20" s="7">
         <v>110000</v>
       </c>
-      <c r="E20" s="6">
+      <c r="E20" s="8">
         <v>2</v>
       </c>
-      <c r="F20" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="G20" s="8" t="str">
-        <f t="shared" si="0"/>
-        <v>Últimas unidades</v>
-      </c>
-      <c r="H20" s="9" t="s">
+      <c r="F20" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="G20" s="10">
+        <f>IF(F20="NO","Oculto",IF(E20&lt;=0,"AGOTADO",IF(E20&lt;=5,"Últimas unidades","Disponible")))</f>
+      </c>
+      <c r="H20" s="11" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="21" spans="1:8" s="2" customFormat="1" ht="12.75" x14ac:dyDescent="0.25">
-      <c r="A21" s="3" t="s">
+    <row r="21" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A21" s="5" t="s">
         <v>50</v>
       </c>
-      <c r="B21" s="4" t="s">
+      <c r="B21" s="6" t="s">
         <v>51</v>
       </c>
-      <c r="C21" s="4" t="s">
+      <c r="C21" s="6" t="s">
         <v>32</v>
       </c>
-      <c r="D21" s="5">
+      <c r="D21" s="7">
         <v>120000</v>
       </c>
-      <c r="E21" s="6">
+      <c r="E21" s="8">
         <v>0</v>
       </c>
-      <c r="F21" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="G21" s="8" t="str">
-        <f t="shared" si="0"/>
-        <v>AGOTADO</v>
-      </c>
-      <c r="H21" s="9" t="s">
+      <c r="F21" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="G21" s="10">
+        <f>IF(F21="NO","Oculto",IF(E21&lt;=0,"AGOTADO",IF(E21&lt;=5,"Últimas unidades","Disponible")))</f>
+      </c>
+      <c r="H21" s="11" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="22" spans="1:8" s="2" customFormat="1" ht="12.75" x14ac:dyDescent="0.25">
-      <c r="A22" s="10" t="s">
+    <row r="22" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A22" s="12" t="s">
         <v>53</v>
       </c>
-      <c r="B22" s="2" t="s">
+      <c r="B22" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="C22" s="2" t="s">
+      <c r="C22" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="D22" s="5">
+      <c r="D22" s="7">
         <v>120000</v>
       </c>
-      <c r="E22" s="6">
+      <c r="E22" s="8">
         <v>0</v>
       </c>
-      <c r="F22" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="G22" s="8" t="str">
-        <f t="shared" si="0"/>
-        <v>AGOTADO</v>
-      </c>
-      <c r="H22" s="9" t="s">
+      <c r="F22" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="G22" s="10">
+        <f>IF(F22="NO","Oculto",IF(E22&lt;=0,"AGOTADO",IF(E22&lt;=5,"Últimas unidades","Disponible")))</f>
+      </c>
+      <c r="H22" s="11" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="23" spans="1:8" s="2" customFormat="1" ht="12.75" x14ac:dyDescent="0.25">
-      <c r="A23" s="3" t="s">
+    <row r="23" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A23" s="5" t="s">
         <v>55</v>
       </c>
-      <c r="B23" s="4" t="s">
+      <c r="B23" s="6" t="s">
         <v>56</v>
       </c>
-      <c r="C23" s="4" t="s">
+      <c r="C23" s="6" t="s">
         <v>32</v>
       </c>
-      <c r="D23" s="5">
+      <c r="D23" s="7">
         <v>140000</v>
       </c>
-      <c r="E23" s="6">
+      <c r="E23" s="8">
         <v>2</v>
       </c>
-      <c r="F23" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="G23" s="8" t="str">
-        <f t="shared" si="0"/>
-        <v>Últimas unidades</v>
-      </c>
-      <c r="H23" s="9" t="s">
+      <c r="F23" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="G23" s="10">
+        <f>IF(F23="NO","Oculto",IF(E23&lt;=0,"AGOTADO",IF(E23&lt;=5,"Últimas unidades","Disponible")))</f>
+      </c>
+      <c r="H23" s="11" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="24" spans="1:8" s="2" customFormat="1" ht="25.5" x14ac:dyDescent="0.25">
-      <c r="A24" s="10" t="s">
+    <row r="24" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A24" s="12" t="s">
         <v>58</v>
       </c>
-      <c r="B24" s="2" t="s">
+      <c r="B24" s="4" t="s">
         <v>59</v>
       </c>
-      <c r="C24" s="2" t="s">
+      <c r="C24" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="D24" s="5">
+      <c r="D24" s="7">
         <v>130000</v>
       </c>
-      <c r="E24" s="6">
+      <c r="E24" s="8">
         <v>1</v>
       </c>
-      <c r="F24" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="G24" s="8" t="str">
-        <f t="shared" si="0"/>
-        <v>Últimas unidades</v>
-      </c>
-      <c r="H24" s="9" t="s">
+      <c r="F24" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="G24" s="10">
+        <f>IF(F24="NO","Oculto",IF(E24&lt;=0,"AGOTADO",IF(E24&lt;=5,"Últimas unidades","Disponible")))</f>
+      </c>
+      <c r="H24" s="11" t="s">
         <v>60</v>
       </c>
     </row>
-    <row r="25" spans="1:8" s="2" customFormat="1" ht="12.75" x14ac:dyDescent="0.25">
-      <c r="A25" s="3" t="s">
+    <row r="25" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A25" s="5" t="s">
         <v>61</v>
       </c>
-      <c r="B25" s="4" t="s">
+      <c r="B25" s="6" t="s">
         <v>22</v>
       </c>
-      <c r="C25" s="4" t="s">
+      <c r="C25" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="D25" s="5">
+      <c r="D25" s="7">
         <v>130000</v>
       </c>
-      <c r="E25" s="6">
+      <c r="E25" s="8">
         <v>1</v>
       </c>
-      <c r="F25" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="G25" s="8" t="str">
-        <f t="shared" si="0"/>
-        <v>Últimas unidades</v>
-      </c>
-      <c r="H25" s="9" t="s">
+      <c r="F25" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="G25" s="10">
+        <f>IF(F25="NO","Oculto",IF(E25&lt;=0,"AGOTADO",IF(E25&lt;=5,"Últimas unidades","Disponible")))</f>
+      </c>
+      <c r="H25" s="11" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="26" spans="1:8" s="2" customFormat="1" ht="12.75" x14ac:dyDescent="0.25">
-      <c r="A26" s="10" t="s">
+    <row r="26" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A26" s="12" t="s">
         <v>63</v>
       </c>
-      <c r="B26" s="2" t="s">
+      <c r="B26" s="4" t="s">
         <v>64</v>
       </c>
-      <c r="C26" s="2" t="s">
+      <c r="C26" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="D26" s="5">
+      <c r="D26" s="7">
         <v>140000</v>
       </c>
-      <c r="E26" s="6">
+      <c r="E26" s="8">
         <v>3</v>
       </c>
-      <c r="F26" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="G26" s="8" t="str">
-        <f t="shared" si="0"/>
-        <v>Últimas unidades</v>
-      </c>
-      <c r="H26" s="9" t="s">
+      <c r="F26" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="G26" s="10">
+        <f>IF(F26="NO","Oculto",IF(E26&lt;=0,"AGOTADO",IF(E26&lt;=5,"Últimas unidades","Disponible")))</f>
+      </c>
+      <c r="H26" s="11" t="s">
         <v>65</v>
       </c>
     </row>
-    <row r="27" spans="1:8" s="2" customFormat="1" ht="12.75" x14ac:dyDescent="0.25">
-      <c r="A27" s="3" t="s">
+    <row r="27" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A27" s="5" t="s">
         <v>66</v>
       </c>
-      <c r="B27" s="4" t="s">
+      <c r="B27" s="6" t="s">
         <v>56</v>
       </c>
-      <c r="C27" s="4" t="s">
+      <c r="C27" s="6" t="s">
         <v>32</v>
       </c>
-      <c r="D27" s="5">
+      <c r="D27" s="7">
         <v>130000</v>
       </c>
-      <c r="E27" s="6">
+      <c r="E27" s="8">
         <v>1</v>
       </c>
-      <c r="F27" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="G27" s="8" t="str">
-        <f t="shared" si="0"/>
-        <v>Últimas unidades</v>
-      </c>
-      <c r="H27" s="9" t="s">
+      <c r="F27" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="G27" s="10">
+        <f>IF(F27="NO","Oculto",IF(E27&lt;=0,"AGOTADO",IF(E27&lt;=5,"Últimas unidades","Disponible")))</f>
+      </c>
+      <c r="H27" s="11" t="s">
         <v>67</v>
       </c>
     </row>
-    <row r="28" spans="1:8" s="2" customFormat="1" ht="25.5" x14ac:dyDescent="0.25">
-      <c r="A28" s="10" t="s">
+    <row r="28" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A28" s="12" t="s">
         <v>68</v>
       </c>
-      <c r="B28" s="2" t="s">
+      <c r="B28" s="4" t="s">
         <v>69</v>
       </c>
-      <c r="C28" s="2" t="s">
+      <c r="C28" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="D28" s="5">
+      <c r="D28" s="7">
         <v>120000</v>
       </c>
-      <c r="E28" s="6">
+      <c r="E28" s="8">
         <v>0</v>
       </c>
-      <c r="F28" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="G28" s="8" t="str">
-        <f t="shared" si="0"/>
-        <v>AGOTADO</v>
-      </c>
-      <c r="H28" s="9" t="s">
+      <c r="F28" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="G28" s="10">
+        <f>IF(F28="NO","Oculto",IF(E28&lt;=0,"AGOTADO",IF(E28&lt;=5,"Últimas unidades","Disponible")))</f>
+      </c>
+      <c r="H28" s="11" t="s">
         <v>70</v>
       </c>
     </row>
-    <row r="29" spans="1:8" s="2" customFormat="1" ht="12.75" x14ac:dyDescent="0.25">
-      <c r="A29" s="3" t="s">
+    <row r="29" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A29" s="5" t="s">
         <v>71</v>
       </c>
-      <c r="B29" s="4" t="s">
+      <c r="B29" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="C29" s="4" t="s">
+      <c r="C29" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="D29" s="5">
+      <c r="D29" s="7">
         <v>140000</v>
       </c>
-      <c r="E29" s="6">
+      <c r="E29" s="8">
         <v>1</v>
       </c>
-      <c r="F29" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="G29" s="8" t="str">
-        <f t="shared" si="0"/>
-        <v>Últimas unidades</v>
-      </c>
-      <c r="H29" s="9" t="s">
+      <c r="F29" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="G29" s="10">
+        <f>IF(F29="NO","Oculto",IF(E29&lt;=0,"AGOTADO",IF(E29&lt;=5,"Últimas unidades","Disponible")))</f>
+      </c>
+      <c r="H29" s="11" t="s">
         <v>72</v>
       </c>
     </row>
-    <row r="30" spans="1:8" s="2" customFormat="1" ht="12.75" x14ac:dyDescent="0.25">
-      <c r="A30" s="10" t="s">
+    <row r="30" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A30" s="12" t="s">
         <v>73</v>
       </c>
-      <c r="B30" s="2" t="s">
+      <c r="B30" s="4" t="s">
         <v>74</v>
       </c>
-      <c r="C30" s="2" t="s">
+      <c r="C30" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="D30" s="5">
+      <c r="D30" s="7">
         <v>160000</v>
       </c>
-      <c r="E30" s="6">
+      <c r="E30" s="8">
         <v>2</v>
       </c>
-      <c r="F30" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="G30" s="8" t="str">
-        <f t="shared" si="0"/>
-        <v>Últimas unidades</v>
-      </c>
-      <c r="H30" s="9" t="s">
+      <c r="F30" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="G30" s="10">
+        <f>IF(F30="NO","Oculto",IF(E30&lt;=0,"AGOTADO",IF(E30&lt;=5,"Últimas unidades","Disponible")))</f>
+      </c>
+      <c r="H30" s="11" t="s">
         <v>75</v>
       </c>
     </row>
-    <row r="31" spans="1:8" s="2" customFormat="1" ht="12.75" x14ac:dyDescent="0.25">
-      <c r="A31" s="3" t="s">
+    <row r="31" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A31" s="5" t="s">
         <v>76</v>
       </c>
-      <c r="B31" s="4" t="s">
+      <c r="B31" s="6" t="s">
         <v>22</v>
       </c>
-      <c r="C31" s="4" t="s">
+      <c r="C31" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="D31" s="5">
+      <c r="D31" s="7">
         <v>60000</v>
       </c>
-      <c r="E31" s="6">
+      <c r="E31" s="8">
         <v>10</v>
       </c>
-      <c r="F31" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="G31" s="8" t="str">
-        <f t="shared" si="0"/>
-        <v>Disponible</v>
-      </c>
-      <c r="H31" s="9" t="s">
+      <c r="F31" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="G31" s="10">
+        <f>IF(F31="NO","Oculto",IF(E31&lt;=0,"AGOTADO",IF(E31&lt;=5,"Últimas unidades","Disponible")))</f>
+      </c>
+      <c r="H31" s="11" t="s">
         <v>77</v>
       </c>
     </row>
-    <row r="32" spans="1:8" s="2" customFormat="1" ht="12.75" x14ac:dyDescent="0.25">
-      <c r="A32" s="10" t="s">
+    <row r="32" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A32" s="12" t="s">
         <v>78</v>
       </c>
-      <c r="B32" s="2" t="s">
+      <c r="B32" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="C32" s="2" t="s">
+      <c r="C32" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="D32" s="5">
+      <c r="D32" s="7">
         <v>160000</v>
       </c>
-      <c r="E32" s="6">
+      <c r="E32" s="8">
         <v>1</v>
       </c>
-      <c r="F32" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="G32" s="8" t="str">
-        <f t="shared" si="0"/>
-        <v>Últimas unidades</v>
-      </c>
-      <c r="H32" s="9" t="s">
+      <c r="F32" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="G32" s="10">
+        <f>IF(F32="NO","Oculto",IF(E32&lt;=0,"AGOTADO",IF(E32&lt;=5,"Últimas unidades","Disponible")))</f>
+      </c>
+      <c r="H32" s="11" t="s">
         <v>79</v>
       </c>
     </row>
+    <row r="33" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A33" s="5" t="s">
+        <v>80</v>
+      </c>
+      <c r="B33" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="C33" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="D33" s="7">
+        <v>260000</v>
+      </c>
+      <c r="E33" s="8">
+        <v>1</v>
+      </c>
+      <c r="F33" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="G33" s="10">
+        <f>IF(F33="NO","Oculto",IF(E33&lt;=0,"AGOTADO",IF(E33&lt;=5,"Últimas unidades","Disponible")))</f>
+      </c>
+      <c r="H33" s="11" t="s">
+        <v>81</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A4:G32" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
+  <autoFilter ref="A4:G33"/>
   <mergeCells count="2">
     <mergeCell ref="A1:G1"/>
     <mergeCell ref="A2:G2"/>
   </mergeCells>
+  <conditionalFormatting sqref="G5:G33">
+    <cfRule type="containsText" dxfId="0" priority="1">
+      <formula>NOT(ISERROR(SEARCH("AGOTADO",G5)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="1" priority="2">
+      <formula>NOT(ISERROR(SEARCH("Últimas",G5)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="2" priority="3">
+      <formula>NOT(ISERROR(SEARCH("Oculto",G5)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="3" priority="4">
+      <formula>NOT(ISERROR(SEARCH("Disponible",G5)))</formula>
+    </cfRule>
+  </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation type="whole" operator="greaterThanOrEqual" showErrorMessage="1" errorTitle="Cantidad inválida" error="Escribe un número entero de 0 en adelante." sqref="E5:E32" xr:uid="{00000000-0002-0000-0000-000000000000}">
+    <dataValidation type="whole" operator="greaterThanOrEqual" showErrorMessage="1" errorTitle="Cantidad inválida" error="Escribe un número entero de 0 en adelante." sqref="E5:E33">
       <formula1>0</formula1>
     </dataValidation>
-    <dataValidation type="list" showErrorMessage="1" errorTitle="Valor inválido" error="Escribe SI o NO." sqref="F5:F32" xr:uid="{00000000-0002-0000-0000-000001000000}">
+    <dataValidation type="list" showErrorMessage="1" errorTitle="Valor inválido" error="Escribe SI o NO." sqref="F5:F33">
       <formula1>"SI,NO"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup fitToHeight="0" orientation="landscape" horizontalDpi="4294967295" verticalDpi="4294967295"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
-      <x14:conditionalFormattings>
-        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="containsText" priority="1" operator="containsText" id="{00000000-000E-0000-0000-000001000000}">
-            <xm:f>NOT(ISERROR(SEARCH("AGOTADO",G5)))</xm:f>
-            <x14:dxf>
-              <font>
-                <color rgb="FF9C0006"/>
-              </font>
-              <fill>
-                <patternFill patternType="solid">
-                  <bgColor rgb="FFFFC7CE"/>
-                </patternFill>
-              </fill>
-            </x14:dxf>
-          </x14:cfRule>
-          <x14:cfRule type="containsText" priority="2" operator="containsText" id="{00000000-000E-0000-0000-000002000000}">
-            <xm:f>NOT(ISERROR(SEARCH("Últimas",G5)))</xm:f>
-            <x14:dxf>
-              <font>
-                <color rgb="FF9C6500"/>
-              </font>
-              <fill>
-                <patternFill patternType="solid">
-                  <bgColor rgb="FFFFEB9C"/>
-                </patternFill>
-              </fill>
-            </x14:dxf>
-          </x14:cfRule>
-          <x14:cfRule type="containsText" priority="3" operator="containsText" id="{00000000-000E-0000-0000-000003000000}">
-            <xm:f>NOT(ISERROR(SEARCH("Oculto",G5)))</xm:f>
-            <x14:dxf>
-              <font>
-                <color rgb="FF6B7472"/>
-              </font>
-              <fill>
-                <patternFill patternType="solid">
-                  <bgColor rgb="FFEDEDED"/>
-                </patternFill>
-              </fill>
-            </x14:dxf>
-          </x14:cfRule>
-          <x14:cfRule type="containsText" priority="4" operator="containsText" id="{00000000-000E-0000-0000-000004000000}">
-            <xm:f>NOT(ISERROR(SEARCH("Disponible",G5)))</xm:f>
-            <x14:dxf>
-              <font>
-                <color rgb="FF006100"/>
-              </font>
-              <fill>
-                <patternFill patternType="solid">
-                  <bgColor rgb="FFC6EFCE"/>
-                </patternFill>
-              </fill>
-            </x14:dxf>
-          </x14:cfRule>
-          <xm:sqref>G5:G32</xm:sqref>
-        </x14:conditionalFormatting>
-      </x14:conditionalFormattings>
-    </ext>
-  </extLst>
+  <pageSetup orientation="landscape" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="0"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:B13"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="38" customWidth="1"/>
     <col min="2" max="2" width="20" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="21" t="s">
-        <v>80</v>
-      </c>
-      <c r="B1" s="21"/>
+    <row r="1" ht="24" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A1" s="13" t="s">
+        <v>82</v>
+      </c>
+      <c r="B1" s="13"/>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A3" s="11" t="s">
-        <v>81</v>
-      </c>
-      <c r="B3" s="12">
-        <f>COUNTA(Inventario!$A$5:$A$32)</f>
-        <v>28</v>
+      <c r="A3" s="14" t="s">
+        <v>83</v>
+      </c>
+      <c r="B3" s="15">
+        <f>COUNTA(Inventario!$A$5:$A$33)</f>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A4" s="11" t="s">
-        <v>82</v>
-      </c>
-      <c r="B4" s="12">
-        <f>COUNTIF(Inventario!$G$5:$G$32,"Disponible")</f>
-        <v>1</v>
+      <c r="A4" s="14" t="s">
+        <v>84</v>
+      </c>
+      <c r="B4" s="15">
+        <f>COUNTIF(Inventario!$G$5:$G$33,"Disponible")</f>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A5" s="11" t="s">
-        <v>83</v>
-      </c>
-      <c r="B5" s="12">
-        <f>COUNTIF(Inventario!$G$5:$G$32,"Últimas unidades")</f>
-        <v>18</v>
+      <c r="A5" s="14" t="s">
+        <v>85</v>
+      </c>
+      <c r="B5" s="15">
+        <f>COUNTIF(Inventario!$G$5:$G$33,"Últimas unidades")</f>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A6" s="11" t="s">
-        <v>84</v>
-      </c>
-      <c r="B6" s="12">
-        <f>COUNTIF(Inventario!$G$5:$G$32,"AGOTADO")</f>
-        <v>9</v>
+      <c r="A6" s="14" t="s">
+        <v>86</v>
+      </c>
+      <c r="B6" s="15">
+        <f>COUNTIF(Inventario!$G$5:$G$33,"AGOTADO")</f>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A7" s="11" t="s">
-        <v>85</v>
-      </c>
-      <c r="B7" s="12">
-        <f>COUNTIF(Inventario!$G$5:$G$32,"Oculto")</f>
-        <v>0</v>
+      <c r="A7" s="14" t="s">
+        <v>87</v>
+      </c>
+      <c r="B7" s="15">
+        <f>COUNTIF(Inventario!$G$5:$G$33,"Oculto")</f>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A8" s="11" t="s">
-        <v>86</v>
-      </c>
-      <c r="B8" s="12">
-        <f>SUM(Inventario!$E$5:$E$32)</f>
-        <v>38</v>
+      <c r="A8" s="14" t="s">
+        <v>88</v>
+      </c>
+      <c r="B8" s="15">
+        <f>SUM(Inventario!$E$5:$E$33)</f>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A9" s="11" t="s">
-        <v>87</v>
-      </c>
-      <c r="B9" s="13">
-        <f>SUMPRODUCT(Inventario!$D$5:$D$32,Inventario!$E$5:$E$32)</f>
-        <v>4450000</v>
-      </c>
-    </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A11" s="14" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A13" s="15" t="s">
+      <c r="A9" s="14" t="s">
         <v>89</v>
+      </c>
+      <c r="B9" s="16">
+        <f>SUMPRODUCT(Inventario!$D$5:$D$33,Inventario!$E$5:$E$33)</f>
+      </c>
+    </row>
+    <row r="11" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A11" s="17" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="13" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A13" s="18" t="s">
+        <v>91</v>
       </c>
     </row>
   </sheetData>
@@ -1932,145 +1852,145 @@
     <mergeCell ref="A1:B1"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:A25"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="110" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="16" t="s">
-        <v>90</v>
+    <row r="1" ht="24" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A1" s="19" t="s">
+        <v>92</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A2" s="10" t="s">
-        <v>91</v>
+      <c r="A2" s="12" t="s">
+        <v>93</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A3" s="10" t="s">
-        <v>92</v>
+      <c r="A3" s="12" t="s">
+        <v>94</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A4" s="10" t="s">
+      <c r="A4" s="12" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A5" s="12" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="6" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A6" s="12" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="7" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A7" s="12" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="8" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A8" s="12" t="s">
         <v>93</v>
       </c>
     </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A5" s="10" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="6" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A6" s="10" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="7" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A7" s="10" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="8" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A8" s="10" t="s">
-        <v>91</v>
-      </c>
-    </row>
     <row r="9" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A9" s="17" t="s">
-        <v>97</v>
+      <c r="A9" s="20" t="s">
+        <v>99</v>
       </c>
     </row>
     <row r="10" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A10" s="10" t="s">
-        <v>98</v>
+      <c r="A10" s="12" t="s">
+        <v>100</v>
       </c>
     </row>
     <row r="11" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A11" s="10" t="s">
-        <v>99</v>
+      <c r="A11" s="12" t="s">
+        <v>101</v>
       </c>
     </row>
     <row r="12" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A12" s="10" t="s">
-        <v>100</v>
+      <c r="A12" s="12" t="s">
+        <v>102</v>
       </c>
     </row>
     <row r="13" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A13" s="10" t="s">
-        <v>101</v>
+      <c r="A13" s="12" t="s">
+        <v>103</v>
       </c>
     </row>
     <row r="14" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A14" s="10" t="s">
-        <v>102</v>
+      <c r="A14" s="12" t="s">
+        <v>104</v>
       </c>
     </row>
     <row r="15" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A15" s="10" t="s">
-        <v>91</v>
+      <c r="A15" s="12" t="s">
+        <v>93</v>
       </c>
     </row>
     <row r="16" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A16" s="17" t="s">
-        <v>103</v>
+      <c r="A16" s="20" t="s">
+        <v>105</v>
       </c>
     </row>
     <row r="17" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A17" s="10" t="s">
-        <v>104</v>
+      <c r="A17" s="12" t="s">
+        <v>106</v>
       </c>
     </row>
     <row r="18" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A18" s="10" t="s">
-        <v>105</v>
+      <c r="A18" s="12" t="s">
+        <v>107</v>
       </c>
     </row>
     <row r="19" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A19" s="10" t="s">
-        <v>106</v>
+      <c r="A19" s="12" t="s">
+        <v>108</v>
       </c>
     </row>
     <row r="20" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A20" s="10" t="s">
-        <v>107</v>
+      <c r="A20" s="12" t="s">
+        <v>109</v>
       </c>
     </row>
     <row r="21" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A21" s="10" t="s">
-        <v>91</v>
+      <c r="A21" s="12" t="s">
+        <v>93</v>
       </c>
     </row>
     <row r="22" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A22" s="17" t="s">
-        <v>108</v>
+      <c r="A22" s="20" t="s">
+        <v>110</v>
       </c>
     </row>
     <row r="23" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A23" s="10" t="s">
-        <v>109</v>
+      <c r="A23" s="12" t="s">
+        <v>111</v>
       </c>
     </row>
     <row r="24" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A24" s="10" t="s">
-        <v>110</v>
+      <c r="A24" s="12" t="s">
+        <v>112</v>
       </c>
     </row>
     <row r="25" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A25" s="10" t="s">
-        <v>111</v>
+      <c r="A25" s="12" t="s">
+        <v>113</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Agregar Creatina Orgain (#30) y Berberina Feel Good (#31), $160.000 c/u, stock 2
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/inventario.xlsx
+++ b/inventario.xlsx
@@ -1,39 +1,19 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="27932"/>
-  <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4B62A83B-C001-4EEF-9CCD-8C2AD915B418}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
-  <bookViews>
-    <workbookView xWindow="20370" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
-  </bookViews>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
+  <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
   <sheets>
-    <sheet name="Inventario" sheetId="1" r:id="rId1"/>
-    <sheet name="Resumen" sheetId="2" r:id="rId2"/>
-    <sheet name="Instrucciones" sheetId="3" r:id="rId3"/>
+    <sheet sheetId="1" name="Inventario" state="visible" r:id="rId4"/>
+    <sheet sheetId="2" name="Resumen" state="visible" r:id="rId5"/>
+    <sheet sheetId="3" name="Instrucciones" state="visible" r:id="rId6"/>
   </sheets>
-  <calcPr calcId="191029"/>
-  <extLst>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
-    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
-      <xlwcv:version setVersion="1"/>
-    </ext>
-  </extLst>
+  <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="190" uniqueCount="114">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="200" uniqueCount="120">
   <si>
     <t>INVENTARIO — El Garaje de Rochi</t>
   </si>
@@ -281,6 +261,24 @@
     <t>SUP-COQ10-140</t>
   </si>
   <si>
+    <t>Orgain Creatina Monohidratada Micronizada sin sabor (675 g)</t>
+  </si>
+  <si>
+    <t>Orgain</t>
+  </si>
+  <si>
+    <t>SUP-CREATINA-675</t>
+  </si>
+  <si>
+    <t>Feel Good Berberina Fitosoma de alta absorción (120 cápsulas veganas)</t>
+  </si>
+  <si>
+    <t>Feel Good Company</t>
+  </si>
+  <si>
+    <t>SUP-BERBER-FG120</t>
+  </si>
+  <si>
     <t>RESUMEN DEL INVENTARIO</t>
   </si>
   <si>
@@ -308,7 +306,7 @@
     <t>Se recalcula solo cuando cambias las cantidades en la hoja Inventario.</t>
   </si>
   <si>
-    <t>Generado: 25/9/2026, 10:55:35 a. m.</t>
+    <t>Generado: 29/10/2026, 9:40:56 a. m.</t>
   </si>
   <si>
     <t>CÓMO USAR ESTE EXCEL</t>
@@ -380,34 +378,34 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="&quot;$&quot;\ #,##0"/>
+    <numFmt numFmtId="164" formatCode="&quot;$&quot; #,##0"/>
   </numFmts>
   <fonts count="13" x14ac:knownFonts="1">
     <font>
-      <sz val="11"/>
       <color theme="1"/>
-      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+      <sz val="11"/>
+      <name val="Calibri"/>
     </font>
     <font>
       <b/>
+      <color rgb="FFFFFFFF"/>
       <sz val="16"/>
-      <color rgb="FFFFFFFF"/>
       <name val="Arial"/>
     </font>
     <font>
       <i/>
+      <color rgb="FF6b7472"/>
       <sz val="9"/>
-      <color rgb="FF6B7472"/>
       <name val="Arial"/>
     </font>
     <font>
       <b/>
+      <color rgb="FFFFFFFF"/>
       <sz val="10"/>
-      <color rgb="FFFFFFFF"/>
       <name val="Arial"/>
     </font>
     <font>
@@ -420,14 +418,14 @@
       <name val="Arial"/>
     </font>
     <font>
+      <color rgb="FF9A9A9A"/>
       <sz val="8"/>
-      <color rgb="FF9A9A9A"/>
       <name val="Arial"/>
     </font>
     <font>
       <b/>
+      <color rgb="FFFFFFFF"/>
       <sz val="14"/>
-      <color rgb="FFFFFFFF"/>
       <name val="Arial"/>
     </font>
     <font>
@@ -440,20 +438,20 @@
       <name val="Arial"/>
     </font>
     <font>
+      <color rgb="FF9A9A9A"/>
       <sz val="9"/>
-      <color rgb="FF9A9A9A"/>
       <name val="Arial"/>
     </font>
     <font>
       <b/>
+      <color rgb="FFFFFFFF"/>
       <sz val="15"/>
-      <color rgb="FFFFFFFF"/>
       <name val="Arial"/>
     </font>
     <font>
       <b/>
+      <color rgb="FF2E8B80"/>
       <sz val="11"/>
-      <color rgb="FF2E8B80"/>
       <name val="Arial"/>
     </font>
   </fonts>
@@ -504,6 +502,12 @@
   </cellStyleXfs>
   <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -534,6 +538,7 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="1" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
@@ -549,13 +554,6 @@
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -563,21 +561,11 @@
   <dxfs count="4">
     <dxf>
       <font>
-        <color rgb="FF006100"/>
+        <color rgb="FF9C0006"/>
       </font>
       <fill>
         <patternFill patternType="solid">
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF6B7472"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFEDEDED"/>
+          <bgColor rgb="FFFFC7CE"/>
         </patternFill>
       </fill>
     </dxf>
@@ -593,11 +581,21 @@
     </dxf>
     <dxf>
       <font>
-        <color rgb="FF9C0006"/>
+        <color rgb="FF6b7472"/>
       </font>
       <fill>
         <patternFill patternType="solid">
-          <bgColor rgb="FFFFC7CE"/>
+          <bgColor rgb="FFEDEDED"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFC6EFCE"/>
         </patternFill>
       </fill>
     </dxf>
@@ -935,12 +933,12 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:H33"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:H35"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="52" customWidth="1"/>
     <col min="2" max="2" width="18" customWidth="1"/>
@@ -951,1003 +949,972 @@
     <col min="7" max="8" width="20" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="18" t="s">
+    <row r="1" ht="28" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="18"/>
-      <c r="C1" s="18"/>
-      <c r="D1" s="18"/>
-      <c r="E1" s="18"/>
-      <c r="F1" s="18"/>
-      <c r="G1" s="18"/>
-    </row>
-    <row r="2" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="19" t="s">
+      <c r="B1" s="1"/>
+      <c r="C1" s="1"/>
+      <c r="D1" s="1"/>
+      <c r="E1" s="1"/>
+      <c r="F1" s="1"/>
+      <c r="G1" s="1"/>
+    </row>
+    <row r="2" ht="30" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="19"/>
-      <c r="C2" s="19"/>
-      <c r="D2" s="19"/>
-      <c r="E2" s="19"/>
-      <c r="F2" s="19"/>
-      <c r="G2" s="19"/>
-    </row>
-    <row r="4" spans="1:8" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="1" t="s">
+      <c r="B2" s="2"/>
+      <c r="C2" s="2"/>
+      <c r="D2" s="2"/>
+      <c r="E2" s="2"/>
+      <c r="F2" s="2"/>
+      <c r="G2" s="2"/>
+    </row>
+    <row r="4" ht="32" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A4" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="1" t="s">
+      <c r="B4" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="C4" s="1" t="s">
+      <c r="C4" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="D4" s="1" t="s">
+      <c r="D4" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="E4" s="1" t="s">
+      <c r="E4" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="F4" s="1" t="s">
+      <c r="F4" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="G4" s="1" t="s">
+      <c r="G4" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="H4" s="1" t="s">
+      <c r="H4" s="3" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="5" spans="1:8" s="2" customFormat="1" ht="12.75" x14ac:dyDescent="0.25">
-      <c r="A5" s="3" t="s">
+    <row r="5" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="B5" s="4" t="s">
+      <c r="B5" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="C5" s="4" t="s">
+      <c r="C5" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="D5" s="5">
+      <c r="D5" s="7">
         <v>170000</v>
       </c>
-      <c r="E5" s="6">
+      <c r="E5" s="8">
         <v>2</v>
       </c>
-      <c r="F5" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="G5" s="8" t="str">
-        <f t="shared" ref="G5:G33" si="0">IF(F5="NO","Oculto",IF(E5&lt;=0,"AGOTADO",IF(E5&lt;=5,"Últimas unidades","Disponible")))</f>
-        <v>Últimas unidades</v>
-      </c>
-      <c r="H5" s="9" t="s">
+      <c r="F5" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="G5" s="10">
+        <f>IF(F5="NO","Oculto",IF(E5&lt;=0,"AGOTADO",IF(E5&lt;=5,"Últimas unidades","Disponible")))</f>
+      </c>
+      <c r="H5" s="11" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="6" spans="1:8" s="2" customFormat="1" ht="12.75" x14ac:dyDescent="0.25">
-      <c r="A6" s="10" t="s">
+    <row r="6" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="12" t="s">
         <v>15</v>
       </c>
-      <c r="B6" s="2" t="s">
+      <c r="B6" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="C6" s="2" t="s">
+      <c r="C6" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="D6" s="5">
+      <c r="D6" s="7">
         <v>130000</v>
       </c>
-      <c r="E6" s="6">
+      <c r="E6" s="8">
         <v>2</v>
       </c>
-      <c r="F6" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="G6" s="8" t="str">
-        <f t="shared" si="0"/>
-        <v>Últimas unidades</v>
-      </c>
-      <c r="H6" s="9" t="s">
+      <c r="F6" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="G6" s="10">
+        <f>IF(F6="NO","Oculto",IF(E6&lt;=0,"AGOTADO",IF(E6&lt;=5,"Últimas unidades","Disponible")))</f>
+      </c>
+      <c r="H6" s="11" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="7" spans="1:8" s="2" customFormat="1" ht="12.75" x14ac:dyDescent="0.25">
-      <c r="A7" s="3" t="s">
+    <row r="7" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="B7" s="4" t="s">
+      <c r="B7" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="C7" s="4" t="s">
+      <c r="C7" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="D7" s="5">
+      <c r="D7" s="7">
         <v>130000</v>
       </c>
-      <c r="E7" s="6">
+      <c r="E7" s="8">
         <v>1</v>
       </c>
-      <c r="F7" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="G7" s="8" t="str">
-        <f t="shared" si="0"/>
-        <v>Últimas unidades</v>
-      </c>
-      <c r="H7" s="9" t="s">
+      <c r="F7" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="G7" s="10">
+        <f>IF(F7="NO","Oculto",IF(E7&lt;=0,"AGOTADO",IF(E7&lt;=5,"Últimas unidades","Disponible")))</f>
+      </c>
+      <c r="H7" s="11" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="8" spans="1:8" s="2" customFormat="1" ht="12.75" x14ac:dyDescent="0.25">
-      <c r="A8" s="10" t="s">
+    <row r="8" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="12" t="s">
         <v>21</v>
       </c>
-      <c r="B8" s="2" t="s">
+      <c r="B8" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="C8" s="2" t="s">
+      <c r="C8" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="D8" s="5">
+      <c r="D8" s="7">
         <v>130000</v>
       </c>
-      <c r="E8" s="6">
+      <c r="E8" s="8">
         <v>1</v>
       </c>
-      <c r="F8" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="G8" s="8" t="str">
-        <f t="shared" si="0"/>
-        <v>Últimas unidades</v>
-      </c>
-      <c r="H8" s="9" t="s">
+      <c r="F8" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="G8" s="10">
+        <f>IF(F8="NO","Oculto",IF(E8&lt;=0,"AGOTADO",IF(E8&lt;=5,"Últimas unidades","Disponible")))</f>
+      </c>
+      <c r="H8" s="11" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="9" spans="1:8" s="2" customFormat="1" ht="25.5" x14ac:dyDescent="0.25">
-      <c r="A9" s="3" t="s">
+    <row r="9" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="5" t="s">
         <v>24</v>
       </c>
-      <c r="B9" s="4" t="s">
+      <c r="B9" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="C9" s="4" t="s">
+      <c r="C9" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="D9" s="5">
+      <c r="D9" s="7">
         <v>160000</v>
       </c>
-      <c r="E9" s="6">
+      <c r="E9" s="8">
         <v>0</v>
       </c>
-      <c r="F9" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="G9" s="8" t="str">
-        <f t="shared" si="0"/>
-        <v>AGOTADO</v>
-      </c>
-      <c r="H9" s="9" t="s">
+      <c r="F9" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="G9" s="10">
+        <f>IF(F9="NO","Oculto",IF(E9&lt;=0,"AGOTADO",IF(E9&lt;=5,"Últimas unidades","Disponible")))</f>
+      </c>
+      <c r="H9" s="11" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="10" spans="1:8" s="2" customFormat="1" ht="12.75" x14ac:dyDescent="0.25">
-      <c r="A10" s="10" t="s">
+    <row r="10" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="12" t="s">
         <v>26</v>
       </c>
-      <c r="B10" s="2" t="s">
+      <c r="B10" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="C10" s="2" t="s">
+      <c r="C10" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="D10" s="5">
+      <c r="D10" s="7">
         <v>130000</v>
       </c>
-      <c r="E10" s="6">
+      <c r="E10" s="8">
         <v>1</v>
       </c>
-      <c r="F10" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="G10" s="8" t="str">
-        <f t="shared" si="0"/>
-        <v>Últimas unidades</v>
-      </c>
-      <c r="H10" s="9" t="s">
+      <c r="F10" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="G10" s="10">
+        <f>IF(F10="NO","Oculto",IF(E10&lt;=0,"AGOTADO",IF(E10&lt;=5,"Últimas unidades","Disponible")))</f>
+      </c>
+      <c r="H10" s="11" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="11" spans="1:8" s="2" customFormat="1" ht="12.75" x14ac:dyDescent="0.25">
-      <c r="A11" s="3" t="s">
+    <row r="11" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="5" t="s">
         <v>28</v>
       </c>
-      <c r="B11" s="4" t="s">
+      <c r="B11" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="C11" s="4" t="s">
+      <c r="C11" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="D11" s="5">
+      <c r="D11" s="7">
         <v>120000</v>
       </c>
-      <c r="E11" s="6">
+      <c r="E11" s="8">
         <v>2</v>
       </c>
-      <c r="F11" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="G11" s="8" t="str">
-        <f t="shared" si="0"/>
-        <v>Últimas unidades</v>
-      </c>
-      <c r="H11" s="9" t="s">
+      <c r="F11" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="G11" s="10">
+        <f>IF(F11="NO","Oculto",IF(E11&lt;=0,"AGOTADO",IF(E11&lt;=5,"Últimas unidades","Disponible")))</f>
+      </c>
+      <c r="H11" s="11" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="12" spans="1:8" s="2" customFormat="1" ht="12.75" x14ac:dyDescent="0.25">
-      <c r="A12" s="10" t="s">
+    <row r="12" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="12" t="s">
         <v>30</v>
       </c>
-      <c r="B12" s="2" t="s">
+      <c r="B12" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="C12" s="2" t="s">
+      <c r="C12" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="D12" s="5">
+      <c r="D12" s="7">
         <v>160000</v>
       </c>
-      <c r="E12" s="6">
+      <c r="E12" s="8">
         <v>0</v>
       </c>
-      <c r="F12" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="G12" s="8" t="str">
-        <f t="shared" si="0"/>
-        <v>AGOTADO</v>
-      </c>
-      <c r="H12" s="9" t="s">
+      <c r="F12" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="G12" s="10">
+        <f>IF(F12="NO","Oculto",IF(E12&lt;=0,"AGOTADO",IF(E12&lt;=5,"Últimas unidades","Disponible")))</f>
+      </c>
+      <c r="H12" s="11" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="13" spans="1:8" s="2" customFormat="1" ht="12.75" x14ac:dyDescent="0.25">
-      <c r="A13" s="3" t="s">
+    <row r="13" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="5" t="s">
         <v>34</v>
       </c>
-      <c r="B13" s="4" t="s">
+      <c r="B13" s="6" t="s">
         <v>31</v>
       </c>
-      <c r="C13" s="4" t="s">
+      <c r="C13" s="6" t="s">
         <v>32</v>
       </c>
-      <c r="D13" s="5">
+      <c r="D13" s="7">
         <v>160000</v>
       </c>
-      <c r="E13" s="6">
+      <c r="E13" s="8">
         <v>0</v>
       </c>
-      <c r="F13" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="G13" s="8" t="str">
-        <f t="shared" si="0"/>
-        <v>AGOTADO</v>
-      </c>
-      <c r="H13" s="9" t="s">
+      <c r="F13" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="G13" s="10">
+        <f>IF(F13="NO","Oculto",IF(E13&lt;=0,"AGOTADO",IF(E13&lt;=5,"Últimas unidades","Disponible")))</f>
+      </c>
+      <c r="H13" s="11" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="14" spans="1:8" s="2" customFormat="1" ht="12.75" x14ac:dyDescent="0.25">
-      <c r="A14" s="10" t="s">
+    <row r="14" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="12" t="s">
         <v>36</v>
       </c>
-      <c r="B14" s="2" t="s">
+      <c r="B14" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="C14" s="2" t="s">
+      <c r="C14" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="D14" s="5">
+      <c r="D14" s="7">
         <v>160000</v>
       </c>
-      <c r="E14" s="6">
+      <c r="E14" s="8">
         <v>0</v>
       </c>
-      <c r="F14" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="G14" s="8" t="str">
-        <f t="shared" si="0"/>
-        <v>AGOTADO</v>
-      </c>
-      <c r="H14" s="9" t="s">
+      <c r="F14" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="G14" s="10">
+        <f>IF(F14="NO","Oculto",IF(E14&lt;=0,"AGOTADO",IF(E14&lt;=5,"Últimas unidades","Disponible")))</f>
+      </c>
+      <c r="H14" s="11" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="15" spans="1:8" s="2" customFormat="1" ht="12.75" x14ac:dyDescent="0.25">
-      <c r="A15" s="3" t="s">
+    <row r="15" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="5" t="s">
         <v>38</v>
       </c>
-      <c r="B15" s="4" t="s">
+      <c r="B15" s="6" t="s">
         <v>31</v>
       </c>
-      <c r="C15" s="4" t="s">
+      <c r="C15" s="6" t="s">
         <v>32</v>
       </c>
-      <c r="D15" s="5">
+      <c r="D15" s="7">
         <v>200000</v>
       </c>
-      <c r="E15" s="6">
+      <c r="E15" s="8">
         <v>0</v>
       </c>
-      <c r="F15" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="G15" s="8" t="str">
-        <f t="shared" si="0"/>
-        <v>AGOTADO</v>
-      </c>
-      <c r="H15" s="9" t="s">
+      <c r="F15" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="G15" s="10">
+        <f>IF(F15="NO","Oculto",IF(E15&lt;=0,"AGOTADO",IF(E15&lt;=5,"Últimas unidades","Disponible")))</f>
+      </c>
+      <c r="H15" s="11" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="16" spans="1:8" s="2" customFormat="1" ht="12.75" x14ac:dyDescent="0.25">
-      <c r="A16" s="10" t="s">
+    <row r="16" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="12" t="s">
         <v>40</v>
       </c>
-      <c r="B16" s="2" t="s">
+      <c r="B16" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="C16" s="2" t="s">
+      <c r="C16" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="D16" s="5">
+      <c r="D16" s="7">
         <v>130000</v>
       </c>
-      <c r="E16" s="6">
+      <c r="E16" s="8">
         <v>0</v>
       </c>
-      <c r="F16" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="G16" s="8" t="str">
-        <f t="shared" si="0"/>
-        <v>AGOTADO</v>
-      </c>
-      <c r="H16" s="9" t="s">
+      <c r="F16" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="G16" s="10">
+        <f>IF(F16="NO","Oculto",IF(E16&lt;=0,"AGOTADO",IF(E16&lt;=5,"Últimas unidades","Disponible")))</f>
+      </c>
+      <c r="H16" s="11" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="17" spans="1:8" s="2" customFormat="1" ht="12.75" x14ac:dyDescent="0.25">
-      <c r="A17" s="3" t="s">
+    <row r="17" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A17" s="5" t="s">
         <v>42</v>
       </c>
-      <c r="B17" s="4" t="s">
+      <c r="B17" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="C17" s="4" t="s">
+      <c r="C17" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="D17" s="5">
+      <c r="D17" s="7">
         <v>200000</v>
       </c>
-      <c r="E17" s="6">
+      <c r="E17" s="8">
         <v>1</v>
       </c>
-      <c r="F17" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="G17" s="8" t="str">
-        <f t="shared" si="0"/>
-        <v>Últimas unidades</v>
-      </c>
-      <c r="H17" s="9" t="s">
+      <c r="F17" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="G17" s="10">
+        <f>IF(F17="NO","Oculto",IF(E17&lt;=0,"AGOTADO",IF(E17&lt;=5,"Últimas unidades","Disponible")))</f>
+      </c>
+      <c r="H17" s="11" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="18" spans="1:8" s="2" customFormat="1" ht="25.5" x14ac:dyDescent="0.25">
-      <c r="A18" s="10" t="s">
+    <row r="18" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A18" s="12" t="s">
         <v>44</v>
       </c>
-      <c r="B18" s="2" t="s">
+      <c r="B18" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="C18" s="2" t="s">
+      <c r="C18" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="D18" s="5">
+      <c r="D18" s="7">
         <v>130000</v>
       </c>
-      <c r="E18" s="6">
+      <c r="E18" s="8">
         <v>0</v>
       </c>
-      <c r="F18" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="G18" s="8" t="str">
-        <f t="shared" si="0"/>
-        <v>AGOTADO</v>
-      </c>
-      <c r="H18" s="9" t="s">
+      <c r="F18" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="G18" s="10">
+        <f>IF(F18="NO","Oculto",IF(E18&lt;=0,"AGOTADO",IF(E18&lt;=5,"Últimas unidades","Disponible")))</f>
+      </c>
+      <c r="H18" s="11" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="19" spans="1:8" s="2" customFormat="1" ht="12.75" x14ac:dyDescent="0.25">
-      <c r="A19" s="3" t="s">
+    <row r="19" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="5" t="s">
         <v>46</v>
       </c>
-      <c r="B19" s="4" t="s">
+      <c r="B19" s="6" t="s">
         <v>22</v>
       </c>
-      <c r="C19" s="4" t="s">
+      <c r="C19" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="D19" s="5">
+      <c r="D19" s="7">
         <v>120000</v>
       </c>
-      <c r="E19" s="6">
+      <c r="E19" s="8">
         <v>4</v>
       </c>
-      <c r="F19" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="G19" s="8" t="str">
-        <f t="shared" si="0"/>
-        <v>Últimas unidades</v>
-      </c>
-      <c r="H19" s="9" t="s">
+      <c r="F19" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="G19" s="10">
+        <f>IF(F19="NO","Oculto",IF(E19&lt;=0,"AGOTADO",IF(E19&lt;=5,"Últimas unidades","Disponible")))</f>
+      </c>
+      <c r="H19" s="11" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="20" spans="1:8" s="2" customFormat="1" ht="12.75" x14ac:dyDescent="0.25">
-      <c r="A20" s="10" t="s">
+    <row r="20" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A20" s="12" t="s">
         <v>48</v>
       </c>
-      <c r="B20" s="2" t="s">
+      <c r="B20" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="C20" s="2" t="s">
+      <c r="C20" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="D20" s="5">
+      <c r="D20" s="7">
         <v>110000</v>
       </c>
-      <c r="E20" s="6">
+      <c r="E20" s="8">
         <v>2</v>
       </c>
-      <c r="F20" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="G20" s="8" t="str">
-        <f t="shared" si="0"/>
-        <v>Últimas unidades</v>
-      </c>
-      <c r="H20" s="9" t="s">
+      <c r="F20" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="G20" s="10">
+        <f>IF(F20="NO","Oculto",IF(E20&lt;=0,"AGOTADO",IF(E20&lt;=5,"Últimas unidades","Disponible")))</f>
+      </c>
+      <c r="H20" s="11" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="21" spans="1:8" s="2" customFormat="1" ht="12.75" x14ac:dyDescent="0.25">
-      <c r="A21" s="3" t="s">
+    <row r="21" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A21" s="5" t="s">
         <v>50</v>
       </c>
-      <c r="B21" s="4" t="s">
+      <c r="B21" s="6" t="s">
         <v>51</v>
       </c>
-      <c r="C21" s="4" t="s">
+      <c r="C21" s="6" t="s">
         <v>32</v>
       </c>
-      <c r="D21" s="5">
+      <c r="D21" s="7">
         <v>120000</v>
       </c>
-      <c r="E21" s="6">
+      <c r="E21" s="8">
         <v>0</v>
       </c>
-      <c r="F21" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="G21" s="8" t="str">
-        <f t="shared" si="0"/>
-        <v>AGOTADO</v>
-      </c>
-      <c r="H21" s="9" t="s">
+      <c r="F21" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="G21" s="10">
+        <f>IF(F21="NO","Oculto",IF(E21&lt;=0,"AGOTADO",IF(E21&lt;=5,"Últimas unidades","Disponible")))</f>
+      </c>
+      <c r="H21" s="11" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="22" spans="1:8" s="2" customFormat="1" ht="12.75" x14ac:dyDescent="0.25">
-      <c r="A22" s="10" t="s">
+    <row r="22" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A22" s="12" t="s">
         <v>53</v>
       </c>
-      <c r="B22" s="2" t="s">
+      <c r="B22" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="C22" s="2" t="s">
+      <c r="C22" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="D22" s="5">
+      <c r="D22" s="7">
         <v>120000</v>
       </c>
-      <c r="E22" s="6">
+      <c r="E22" s="8">
         <v>0</v>
       </c>
-      <c r="F22" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="G22" s="8" t="str">
-        <f t="shared" si="0"/>
-        <v>AGOTADO</v>
-      </c>
-      <c r="H22" s="9" t="s">
+      <c r="F22" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="G22" s="10">
+        <f>IF(F22="NO","Oculto",IF(E22&lt;=0,"AGOTADO",IF(E22&lt;=5,"Últimas unidades","Disponible")))</f>
+      </c>
+      <c r="H22" s="11" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="23" spans="1:8" s="2" customFormat="1" ht="12.75" x14ac:dyDescent="0.25">
-      <c r="A23" s="3" t="s">
+    <row r="23" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A23" s="5" t="s">
         <v>55</v>
       </c>
-      <c r="B23" s="4" t="s">
+      <c r="B23" s="6" t="s">
         <v>56</v>
       </c>
-      <c r="C23" s="4" t="s">
+      <c r="C23" s="6" t="s">
         <v>32</v>
       </c>
-      <c r="D23" s="5">
+      <c r="D23" s="7">
         <v>140000</v>
       </c>
-      <c r="E23" s="6">
+      <c r="E23" s="8">
         <v>2</v>
       </c>
-      <c r="F23" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="G23" s="8" t="str">
-        <f t="shared" si="0"/>
-        <v>Últimas unidades</v>
-      </c>
-      <c r="H23" s="9" t="s">
+      <c r="F23" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="G23" s="10">
+        <f>IF(F23="NO","Oculto",IF(E23&lt;=0,"AGOTADO",IF(E23&lt;=5,"Últimas unidades","Disponible")))</f>
+      </c>
+      <c r="H23" s="11" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="24" spans="1:8" s="2" customFormat="1" ht="25.5" x14ac:dyDescent="0.25">
-      <c r="A24" s="10" t="s">
+    <row r="24" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A24" s="12" t="s">
         <v>58</v>
       </c>
-      <c r="B24" s="2" t="s">
+      <c r="B24" s="4" t="s">
         <v>59</v>
       </c>
-      <c r="C24" s="2" t="s">
+      <c r="C24" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="D24" s="5">
+      <c r="D24" s="7">
         <v>130000</v>
       </c>
-      <c r="E24" s="6">
+      <c r="E24" s="8">
         <v>1</v>
       </c>
-      <c r="F24" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="G24" s="8" t="str">
-        <f t="shared" si="0"/>
-        <v>Últimas unidades</v>
-      </c>
-      <c r="H24" s="9" t="s">
+      <c r="F24" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="G24" s="10">
+        <f>IF(F24="NO","Oculto",IF(E24&lt;=0,"AGOTADO",IF(E24&lt;=5,"Últimas unidades","Disponible")))</f>
+      </c>
+      <c r="H24" s="11" t="s">
         <v>60</v>
       </c>
     </row>
-    <row r="25" spans="1:8" s="2" customFormat="1" ht="12.75" x14ac:dyDescent="0.25">
-      <c r="A25" s="3" t="s">
+    <row r="25" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A25" s="5" t="s">
         <v>61</v>
       </c>
-      <c r="B25" s="4" t="s">
+      <c r="B25" s="6" t="s">
         <v>22</v>
       </c>
-      <c r="C25" s="4" t="s">
+      <c r="C25" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="D25" s="5">
+      <c r="D25" s="7">
         <v>130000</v>
       </c>
-      <c r="E25" s="6">
+      <c r="E25" s="8">
         <v>1</v>
       </c>
-      <c r="F25" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="G25" s="8" t="str">
-        <f t="shared" si="0"/>
-        <v>Últimas unidades</v>
-      </c>
-      <c r="H25" s="9" t="s">
+      <c r="F25" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="G25" s="10">
+        <f>IF(F25="NO","Oculto",IF(E25&lt;=0,"AGOTADO",IF(E25&lt;=5,"Últimas unidades","Disponible")))</f>
+      </c>
+      <c r="H25" s="11" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="26" spans="1:8" s="2" customFormat="1" ht="12.75" x14ac:dyDescent="0.25">
-      <c r="A26" s="10" t="s">
+    <row r="26" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A26" s="12" t="s">
         <v>63</v>
       </c>
-      <c r="B26" s="2" t="s">
+      <c r="B26" s="4" t="s">
         <v>64</v>
       </c>
-      <c r="C26" s="2" t="s">
+      <c r="C26" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="D26" s="5">
+      <c r="D26" s="7">
         <v>140000</v>
       </c>
-      <c r="E26" s="6">
+      <c r="E26" s="8">
         <v>3</v>
       </c>
-      <c r="F26" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="G26" s="8" t="str">
-        <f t="shared" si="0"/>
-        <v>Últimas unidades</v>
-      </c>
-      <c r="H26" s="9" t="s">
+      <c r="F26" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="G26" s="10">
+        <f>IF(F26="NO","Oculto",IF(E26&lt;=0,"AGOTADO",IF(E26&lt;=5,"Últimas unidades","Disponible")))</f>
+      </c>
+      <c r="H26" s="11" t="s">
         <v>65</v>
       </c>
     </row>
-    <row r="27" spans="1:8" s="2" customFormat="1" ht="12.75" x14ac:dyDescent="0.25">
-      <c r="A27" s="3" t="s">
+    <row r="27" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A27" s="5" t="s">
         <v>66</v>
       </c>
-      <c r="B27" s="4" t="s">
+      <c r="B27" s="6" t="s">
         <v>56</v>
       </c>
-      <c r="C27" s="4" t="s">
+      <c r="C27" s="6" t="s">
         <v>32</v>
       </c>
-      <c r="D27" s="5">
+      <c r="D27" s="7">
         <v>130000</v>
       </c>
-      <c r="E27" s="6">
+      <c r="E27" s="8">
         <v>1</v>
       </c>
-      <c r="F27" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="G27" s="8" t="str">
-        <f t="shared" si="0"/>
-        <v>Últimas unidades</v>
-      </c>
-      <c r="H27" s="9" t="s">
+      <c r="F27" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="G27" s="10">
+        <f>IF(F27="NO","Oculto",IF(E27&lt;=0,"AGOTADO",IF(E27&lt;=5,"Últimas unidades","Disponible")))</f>
+      </c>
+      <c r="H27" s="11" t="s">
         <v>67</v>
       </c>
     </row>
-    <row r="28" spans="1:8" s="2" customFormat="1" ht="25.5" x14ac:dyDescent="0.25">
-      <c r="A28" s="10" t="s">
+    <row r="28" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A28" s="12" t="s">
         <v>68</v>
       </c>
-      <c r="B28" s="2" t="s">
+      <c r="B28" s="4" t="s">
         <v>69</v>
       </c>
-      <c r="C28" s="2" t="s">
+      <c r="C28" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="D28" s="5">
+      <c r="D28" s="7">
         <v>120000</v>
       </c>
-      <c r="E28" s="6">
+      <c r="E28" s="8">
         <v>0</v>
       </c>
-      <c r="F28" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="G28" s="8" t="str">
-        <f t="shared" si="0"/>
-        <v>AGOTADO</v>
-      </c>
-      <c r="H28" s="9" t="s">
+      <c r="F28" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="G28" s="10">
+        <f>IF(F28="NO","Oculto",IF(E28&lt;=0,"AGOTADO",IF(E28&lt;=5,"Últimas unidades","Disponible")))</f>
+      </c>
+      <c r="H28" s="11" t="s">
         <v>70</v>
       </c>
     </row>
-    <row r="29" spans="1:8" s="2" customFormat="1" ht="12.75" x14ac:dyDescent="0.25">
-      <c r="A29" s="3" t="s">
+    <row r="29" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A29" s="5" t="s">
         <v>71</v>
       </c>
-      <c r="B29" s="4" t="s">
+      <c r="B29" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="C29" s="4" t="s">
+      <c r="C29" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="D29" s="5">
+      <c r="D29" s="7">
         <v>140000</v>
       </c>
-      <c r="E29" s="6">
+      <c r="E29" s="8">
         <v>1</v>
       </c>
-      <c r="F29" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="G29" s="8" t="str">
-        <f t="shared" si="0"/>
-        <v>Últimas unidades</v>
-      </c>
-      <c r="H29" s="9" t="s">
+      <c r="F29" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="G29" s="10">
+        <f>IF(F29="NO","Oculto",IF(E29&lt;=0,"AGOTADO",IF(E29&lt;=5,"Últimas unidades","Disponible")))</f>
+      </c>
+      <c r="H29" s="11" t="s">
         <v>72</v>
       </c>
     </row>
-    <row r="30" spans="1:8" s="2" customFormat="1" ht="12.75" x14ac:dyDescent="0.25">
-      <c r="A30" s="10" t="s">
+    <row r="30" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A30" s="12" t="s">
         <v>73</v>
       </c>
-      <c r="B30" s="2" t="s">
+      <c r="B30" s="4" t="s">
         <v>74</v>
       </c>
-      <c r="C30" s="2" t="s">
+      <c r="C30" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="D30" s="5">
+      <c r="D30" s="7">
         <v>160000</v>
       </c>
-      <c r="E30" s="6">
+      <c r="E30" s="8">
         <v>2</v>
       </c>
-      <c r="F30" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="G30" s="8" t="str">
-        <f t="shared" si="0"/>
-        <v>Últimas unidades</v>
-      </c>
-      <c r="H30" s="9" t="s">
+      <c r="F30" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="G30" s="10">
+        <f>IF(F30="NO","Oculto",IF(E30&lt;=0,"AGOTADO",IF(E30&lt;=5,"Últimas unidades","Disponible")))</f>
+      </c>
+      <c r="H30" s="11" t="s">
         <v>75</v>
       </c>
     </row>
-    <row r="31" spans="1:8" s="2" customFormat="1" ht="12.75" x14ac:dyDescent="0.25">
-      <c r="A31" s="3" t="s">
+    <row r="31" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A31" s="5" t="s">
         <v>76</v>
       </c>
-      <c r="B31" s="4" t="s">
+      <c r="B31" s="6" t="s">
         <v>22</v>
       </c>
-      <c r="C31" s="4" t="s">
+      <c r="C31" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="D31" s="5">
+      <c r="D31" s="7">
         <v>60000</v>
       </c>
-      <c r="E31" s="6">
+      <c r="E31" s="8">
         <v>10</v>
       </c>
-      <c r="F31" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="G31" s="8" t="str">
-        <f t="shared" si="0"/>
-        <v>Disponible</v>
-      </c>
-      <c r="H31" s="9" t="s">
+      <c r="F31" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="G31" s="10">
+        <f>IF(F31="NO","Oculto",IF(E31&lt;=0,"AGOTADO",IF(E31&lt;=5,"Últimas unidades","Disponible")))</f>
+      </c>
+      <c r="H31" s="11" t="s">
         <v>77</v>
       </c>
     </row>
-    <row r="32" spans="1:8" s="2" customFormat="1" ht="12.75" x14ac:dyDescent="0.25">
-      <c r="A32" s="10" t="s">
+    <row r="32" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A32" s="12" t="s">
         <v>78</v>
       </c>
-      <c r="B32" s="2" t="s">
+      <c r="B32" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="C32" s="2" t="s">
+      <c r="C32" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="D32" s="5">
+      <c r="D32" s="7">
         <v>160000</v>
       </c>
-      <c r="E32" s="6">
+      <c r="E32" s="8">
         <v>1</v>
       </c>
-      <c r="F32" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="G32" s="8" t="str">
-        <f t="shared" si="0"/>
-        <v>Últimas unidades</v>
-      </c>
-      <c r="H32" s="9" t="s">
+      <c r="F32" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="G32" s="10">
+        <f>IF(F32="NO","Oculto",IF(E32&lt;=0,"AGOTADO",IF(E32&lt;=5,"Últimas unidades","Disponible")))</f>
+      </c>
+      <c r="H32" s="11" t="s">
         <v>79</v>
       </c>
     </row>
-    <row r="33" spans="1:8" s="2" customFormat="1" ht="12.75" x14ac:dyDescent="0.25">
-      <c r="A33" s="3" t="s">
+    <row r="33" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A33" s="5" t="s">
         <v>80</v>
       </c>
-      <c r="B33" s="4" t="s">
+      <c r="B33" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="C33" s="4" t="s">
+      <c r="C33" s="6" t="s">
         <v>32</v>
       </c>
-      <c r="D33" s="5">
+      <c r="D33" s="7">
         <v>260000</v>
       </c>
-      <c r="E33" s="6">
+      <c r="E33" s="8">
         <v>1</v>
       </c>
-      <c r="F33" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="G33" s="8" t="str">
-        <f t="shared" si="0"/>
-        <v>Últimas unidades</v>
-      </c>
-      <c r="H33" s="9" t="s">
+      <c r="F33" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="G33" s="10">
+        <f>IF(F33="NO","Oculto",IF(E33&lt;=0,"AGOTADO",IF(E33&lt;=5,"Últimas unidades","Disponible")))</f>
+      </c>
+      <c r="H33" s="11" t="s">
         <v>81</v>
       </c>
     </row>
+    <row r="34" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A34" s="12" t="s">
+        <v>82</v>
+      </c>
+      <c r="B34" s="4" t="s">
+        <v>83</v>
+      </c>
+      <c r="C34" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="D34" s="7">
+        <v>160000</v>
+      </c>
+      <c r="E34" s="8">
+        <v>2</v>
+      </c>
+      <c r="F34" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="G34" s="10">
+        <f>IF(F34="NO","Oculto",IF(E34&lt;=0,"AGOTADO",IF(E34&lt;=5,"Últimas unidades","Disponible")))</f>
+      </c>
+      <c r="H34" s="11" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="35" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A35" s="5" t="s">
+        <v>85</v>
+      </c>
+      <c r="B35" s="6" t="s">
+        <v>86</v>
+      </c>
+      <c r="C35" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="D35" s="7">
+        <v>160000</v>
+      </c>
+      <c r="E35" s="8">
+        <v>2</v>
+      </c>
+      <c r="F35" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="G35" s="10">
+        <f>IF(F35="NO","Oculto",IF(E35&lt;=0,"AGOTADO",IF(E35&lt;=5,"Últimas unidades","Disponible")))</f>
+      </c>
+      <c r="H35" s="11" t="s">
+        <v>87</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A4:G33" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
+  <autoFilter ref="A4:G35"/>
   <mergeCells count="2">
     <mergeCell ref="A1:G1"/>
     <mergeCell ref="A2:G2"/>
   </mergeCells>
+  <conditionalFormatting sqref="G5:G35">
+    <cfRule type="containsText" dxfId="0" priority="1">
+      <formula>NOT(ISERROR(SEARCH("AGOTADO",G5)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="1" priority="2">
+      <formula>NOT(ISERROR(SEARCH("Últimas",G5)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="2" priority="3">
+      <formula>NOT(ISERROR(SEARCH("Oculto",G5)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="3" priority="4">
+      <formula>NOT(ISERROR(SEARCH("Disponible",G5)))</formula>
+    </cfRule>
+  </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation type="whole" operator="greaterThanOrEqual" showErrorMessage="1" errorTitle="Cantidad inválida" error="Escribe un número entero de 0 en adelante." sqref="E5:E33" xr:uid="{00000000-0002-0000-0000-000000000000}">
+    <dataValidation type="whole" operator="greaterThanOrEqual" showErrorMessage="1" errorTitle="Cantidad inválida" error="Escribe un número entero de 0 en adelante." sqref="E5:E35">
       <formula1>0</formula1>
     </dataValidation>
-    <dataValidation type="list" showErrorMessage="1" errorTitle="Valor inválido" error="Escribe SI o NO." sqref="F5:F33" xr:uid="{00000000-0002-0000-0000-000001000000}">
+    <dataValidation type="list" showErrorMessage="1" errorTitle="Valor inválido" error="Escribe SI o NO." sqref="F5:F35">
       <formula1>"SI,NO"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup fitToHeight="0" orientation="landscape" horizontalDpi="4294967295" verticalDpi="4294967295"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
-      <x14:conditionalFormattings>
-        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="containsText" priority="1" operator="containsText" id="{00000000-000E-0000-0000-000001000000}">
-            <xm:f>NOT(ISERROR(SEARCH("AGOTADO",G5)))</xm:f>
-            <x14:dxf>
-              <font>
-                <color rgb="FF9C0006"/>
-              </font>
-              <fill>
-                <patternFill patternType="solid">
-                  <bgColor rgb="FFFFC7CE"/>
-                </patternFill>
-              </fill>
-            </x14:dxf>
-          </x14:cfRule>
-          <x14:cfRule type="containsText" priority="2" operator="containsText" id="{00000000-000E-0000-0000-000002000000}">
-            <xm:f>NOT(ISERROR(SEARCH("Últimas",G5)))</xm:f>
-            <x14:dxf>
-              <font>
-                <color rgb="FF9C6500"/>
-              </font>
-              <fill>
-                <patternFill patternType="solid">
-                  <bgColor rgb="FFFFEB9C"/>
-                </patternFill>
-              </fill>
-            </x14:dxf>
-          </x14:cfRule>
-          <x14:cfRule type="containsText" priority="3" operator="containsText" id="{00000000-000E-0000-0000-000003000000}">
-            <xm:f>NOT(ISERROR(SEARCH("Oculto",G5)))</xm:f>
-            <x14:dxf>
-              <font>
-                <color rgb="FF6B7472"/>
-              </font>
-              <fill>
-                <patternFill patternType="solid">
-                  <bgColor rgb="FFEDEDED"/>
-                </patternFill>
-              </fill>
-            </x14:dxf>
-          </x14:cfRule>
-          <x14:cfRule type="containsText" priority="4" operator="containsText" id="{00000000-000E-0000-0000-000004000000}">
-            <xm:f>NOT(ISERROR(SEARCH("Disponible",G5)))</xm:f>
-            <x14:dxf>
-              <font>
-                <color rgb="FF006100"/>
-              </font>
-              <fill>
-                <patternFill patternType="solid">
-                  <bgColor rgb="FFC6EFCE"/>
-                </patternFill>
-              </fill>
-            </x14:dxf>
-          </x14:cfRule>
-          <xm:sqref>G5:G33</xm:sqref>
-        </x14:conditionalFormatting>
-      </x14:conditionalFormattings>
-    </ext>
-  </extLst>
+  <pageSetup orientation="landscape" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="0"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:B13"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="38" customWidth="1"/>
     <col min="2" max="2" width="20" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="20" t="s">
-        <v>82</v>
-      </c>
-      <c r="B1" s="20"/>
+    <row r="1" ht="24" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A1" s="13" t="s">
+        <v>88</v>
+      </c>
+      <c r="B1" s="13"/>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A3" s="11" t="s">
-        <v>83</v>
-      </c>
-      <c r="B3" s="12">
-        <f>COUNTA(Inventario!$A$5:$A$33)</f>
-        <v>29</v>
+      <c r="A3" s="14" t="s">
+        <v>89</v>
+      </c>
+      <c r="B3" s="15">
+        <f>COUNTA(Inventario!$A$5:$A$35)</f>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A4" s="11" t="s">
-        <v>84</v>
-      </c>
-      <c r="B4" s="12">
-        <f>COUNTIF(Inventario!$G$5:$G$33,"Disponible")</f>
-        <v>1</v>
+      <c r="A4" s="14" t="s">
+        <v>90</v>
+      </c>
+      <c r="B4" s="15">
+        <f>COUNTIF(Inventario!$G$5:$G$35,"Disponible")</f>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A5" s="11" t="s">
-        <v>85</v>
-      </c>
-      <c r="B5" s="12">
-        <f>COUNTIF(Inventario!$G$5:$G$33,"Últimas unidades")</f>
-        <v>18</v>
+      <c r="A5" s="14" t="s">
+        <v>91</v>
+      </c>
+      <c r="B5" s="15">
+        <f>COUNTIF(Inventario!$G$5:$G$35,"Últimas unidades")</f>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A6" s="11" t="s">
-        <v>86</v>
-      </c>
-      <c r="B6" s="12">
-        <f>COUNTIF(Inventario!$G$5:$G$33,"AGOTADO")</f>
-        <v>10</v>
+      <c r="A6" s="14" t="s">
+        <v>92</v>
+      </c>
+      <c r="B6" s="15">
+        <f>COUNTIF(Inventario!$G$5:$G$35,"AGOTADO")</f>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A7" s="11" t="s">
-        <v>87</v>
-      </c>
-      <c r="B7" s="12">
-        <f>COUNTIF(Inventario!$G$5:$G$33,"Oculto")</f>
-        <v>0</v>
+      <c r="A7" s="14" t="s">
+        <v>93</v>
+      </c>
+      <c r="B7" s="15">
+        <f>COUNTIF(Inventario!$G$5:$G$35,"Oculto")</f>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A8" s="11" t="s">
-        <v>88</v>
-      </c>
-      <c r="B8" s="12">
-        <f>SUM(Inventario!$E$5:$E$33)</f>
-        <v>39</v>
+      <c r="A8" s="14" t="s">
+        <v>94</v>
+      </c>
+      <c r="B8" s="15">
+        <f>SUM(Inventario!$E$5:$E$35)</f>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A9" s="11" t="s">
-        <v>89</v>
-      </c>
-      <c r="B9" s="13">
-        <f>SUMPRODUCT(Inventario!$D$5:$D$33,Inventario!$E$5:$E$33)</f>
-        <v>4700000</v>
-      </c>
-    </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A11" s="14" t="s">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A13" s="15" t="s">
-        <v>91</v>
+      <c r="A9" s="14" t="s">
+        <v>95</v>
+      </c>
+      <c r="B9" s="16">
+        <f>SUMPRODUCT(Inventario!$D$5:$D$35,Inventario!$E$5:$E$35)</f>
+      </c>
+    </row>
+    <row r="11" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A11" s="17" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="13" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A13" s="18" t="s">
+        <v>97</v>
       </c>
     </row>
   </sheetData>
@@ -1955,145 +1922,145 @@
     <mergeCell ref="A1:B1"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:A25"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="110" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="16" t="s">
-        <v>92</v>
+    <row r="1" ht="24" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A1" s="19" t="s">
+        <v>98</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A2" s="10" t="s">
-        <v>93</v>
+      <c r="A2" s="12" t="s">
+        <v>99</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A3" s="10" t="s">
-        <v>94</v>
+      <c r="A3" s="12" t="s">
+        <v>100</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A4" s="10" t="s">
-        <v>95</v>
+      <c r="A4" s="12" t="s">
+        <v>101</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A5" s="10" t="s">
-        <v>96</v>
+      <c r="A5" s="12" t="s">
+        <v>102</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A6" s="10" t="s">
-        <v>97</v>
+      <c r="A6" s="12" t="s">
+        <v>103</v>
       </c>
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A7" s="10" t="s">
-        <v>98</v>
+      <c r="A7" s="12" t="s">
+        <v>104</v>
       </c>
     </row>
     <row r="8" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A8" s="10" t="s">
-        <v>93</v>
+      <c r="A8" s="12" t="s">
+        <v>99</v>
       </c>
     </row>
     <row r="9" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A9" s="17" t="s">
+      <c r="A9" s="20" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="10" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A10" s="12" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="11" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A11" s="12" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="12" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A12" s="12" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="13" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A13" s="12" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="14" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A14" s="12" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="15" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A15" s="12" t="s">
         <v>99</v>
       </c>
     </row>
-    <row r="10" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A10" s="10" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="11" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A11" s="10" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="12" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A12" s="10" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="13" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A13" s="10" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="14" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A14" s="10" t="s">
-        <v>104</v>
-      </c>
-    </row>
-    <row r="15" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A15" s="10" t="s">
-        <v>93</v>
-      </c>
-    </row>
     <row r="16" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A16" s="17" t="s">
-        <v>105</v>
+      <c r="A16" s="20" t="s">
+        <v>111</v>
       </c>
     </row>
     <row r="17" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A17" s="10" t="s">
-        <v>106</v>
+      <c r="A17" s="12" t="s">
+        <v>112</v>
       </c>
     </row>
     <row r="18" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A18" s="10" t="s">
-        <v>107</v>
+      <c r="A18" s="12" t="s">
+        <v>113</v>
       </c>
     </row>
     <row r="19" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A19" s="10" t="s">
-        <v>108</v>
+      <c r="A19" s="12" t="s">
+        <v>114</v>
       </c>
     </row>
     <row r="20" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A20" s="10" t="s">
-        <v>109</v>
+      <c r="A20" s="12" t="s">
+        <v>115</v>
       </c>
     </row>
     <row r="21" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A21" s="10" t="s">
-        <v>93</v>
+      <c r="A21" s="12" t="s">
+        <v>99</v>
       </c>
     </row>
     <row r="22" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A22" s="17" t="s">
-        <v>110</v>
+      <c r="A22" s="20" t="s">
+        <v>116</v>
       </c>
     </row>
     <row r="23" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A23" s="10" t="s">
-        <v>111</v>
+      <c r="A23" s="12" t="s">
+        <v>117</v>
       </c>
     </row>
     <row r="24" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A24" s="10" t="s">
-        <v>112</v>
+      <c r="A24" s="12" t="s">
+        <v>118</v>
       </c>
     </row>
     <row r="25" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A25" s="10" t="s">
-        <v>113</v>
+      <c r="A25" s="12" t="s">
+        <v>119</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Inventario ordenado alfabeticamente por nombre
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/inventario.xlsx
+++ b/inventario.xlsx
@@ -45,240 +45,240 @@
     <t>SKU — no tocar</t>
   </si>
   <si>
+    <t>Carlyle Panax Ginseng + Ginkgo Biloba 5.000 mg (120 cápsulas)</t>
+  </si>
+  <si>
+    <t>Carlyle</t>
+  </si>
+  <si>
+    <t>Suplementos</t>
+  </si>
+  <si>
+    <t>SI</t>
+  </si>
+  <si>
+    <t>SUP-GINSENG-120</t>
+  </si>
+  <si>
+    <t>Feel Good Berberina Fitosoma de alta absorción (120 cápsulas veganas)</t>
+  </si>
+  <si>
+    <t>Feel Good Company</t>
+  </si>
+  <si>
+    <t>SUP-BERBER-FG120</t>
+  </si>
+  <si>
+    <t>Force Factor Ultra Berberina 1200 mg (60 cápsulas)</t>
+  </si>
+  <si>
+    <t>Force Factor</t>
+  </si>
+  <si>
+    <t>SUP-BERBER-60</t>
+  </si>
+  <si>
+    <t>Kirkland B-12 5000 mcg Disolución Rápida (300 tabletas)</t>
+  </si>
+  <si>
+    <t>Kirkland Signature</t>
+  </si>
+  <si>
+    <t>Vitaminas &amp; Minerales</t>
+  </si>
+  <si>
+    <t>VM-B12-300</t>
+  </si>
+  <si>
+    <t>Kirkland Calcio 600 mg con Vitamina D3 (500 tabletas)</t>
+  </si>
+  <si>
+    <t>VM-CALCIO-500</t>
+  </si>
+  <si>
+    <t>Kirkland Glucosamina y Condroitina (280 tabletas)</t>
+  </si>
+  <si>
+    <t>SUP-GLUCO-280</t>
+  </si>
+  <si>
+    <t>Kirkland Minoxidil 5% para hombres (tubo 60 mL)</t>
+  </si>
+  <si>
+    <t>Cuidado Personal</t>
+  </si>
+  <si>
+    <t>CP-MINOXIDIL</t>
+  </si>
+  <si>
+    <t>Kirkland Omega-3 Aceite de Pescado 1000 mg (400 softgels)</t>
+  </si>
+  <si>
+    <t>SUP-FISHOIL-400</t>
+  </si>
+  <si>
+    <t>Kirkland Super B-Complex con Electrolitos (500 tabletas)</t>
+  </si>
+  <si>
+    <t>VM-SUPERB-500</t>
+  </si>
+  <si>
+    <t>Kirkland Vitamina C Masticable 500 mg (500 tabletas)</t>
+  </si>
+  <si>
+    <t>VM-VITC-500</t>
+  </si>
+  <si>
+    <t>Kirkland Vitamina E 180 mg (500 softgels)</t>
+  </si>
+  <si>
+    <t>VM-VITE-500</t>
+  </si>
+  <si>
+    <t>Natrol Melatonina 5 mg Disolución Rápida (250 tabletas)</t>
+  </si>
+  <si>
+    <t>Natrol</t>
+  </si>
+  <si>
+    <t>SUP-MELA-250</t>
+  </si>
+  <si>
+    <t>Nature Made CoQ10 200 mg (140 softgels)</t>
+  </si>
+  <si>
+    <t>Nature Made</t>
+  </si>
+  <si>
+    <t>SUP-COQ10-140</t>
+  </si>
+  <si>
     <t>Nature Made Magnesio Citrato 250 mg (180 softgels)</t>
   </si>
   <si>
-    <t>Nature Made</t>
-  </si>
-  <si>
-    <t>Vitaminas &amp; Minerales</t>
-  </si>
-  <si>
-    <t>SI</t>
-  </si>
-  <si>
     <t>VM-MAGCIT-180</t>
   </si>
   <si>
+    <t>Nature Made Magnesio Glicinato 100 mg (90 gomitas)</t>
+  </si>
+  <si>
+    <t>VM-MAGGUM-90</t>
+  </si>
+  <si>
+    <t>Nature Made Prenatal Ácido Fólico + DHA (150 softgels)</t>
+  </si>
+  <si>
+    <t>VM-PRENATAL-150</t>
+  </si>
+  <si>
+    <t>Nature Made Vitamina C Extra Fuerte 1000 mg (365 tabletas)</t>
+  </si>
+  <si>
+    <t>VM-VITC-XS-365</t>
+  </si>
+  <si>
+    <t>Nature Made Vitamina D3 25 mcg (650 softgels)</t>
+  </si>
+  <si>
+    <t>VM-VITD3-650</t>
+  </si>
+  <si>
+    <t>Nature's Bounty Hair, Skin &amp; Nails (250 softgels)</t>
+  </si>
+  <si>
+    <t>Nature's Bounty</t>
+  </si>
+  <si>
+    <t>CP-HSN-250</t>
+  </si>
+  <si>
+    <t>Nature's Bounty Hair, Skin &amp; Nails Advanced (230 gomitas)</t>
+  </si>
+  <si>
+    <t>CP-HSN-ADV-230</t>
+  </si>
+  <si>
     <t>Nature's Bounty Magnesio Glicinato 240 mg (180 cápsulas)</t>
   </si>
   <si>
-    <t>Nature's Bounty</t>
-  </si>
-  <si>
     <t>VM-MAGGLY-180</t>
   </si>
   <si>
-    <t>Nature's Bounty Hair, Skin &amp; Nails Advanced (230 gomitas)</t>
-  </si>
-  <si>
-    <t>Cuidado Personal</t>
-  </si>
-  <si>
-    <t>CP-HSN-ADV-230</t>
-  </si>
-  <si>
-    <t>Kirkland Super B-Complex con Electrolitos (500 tabletas)</t>
-  </si>
-  <si>
-    <t>Kirkland Signature</t>
-  </si>
-  <si>
-    <t>VM-SUPERB-500</t>
-  </si>
-  <si>
-    <t>Nature Made Vitamina C Extra Fuerte 1000 mg (365 tabletas)</t>
-  </si>
-  <si>
-    <t>VM-VITC-XS-365</t>
-  </si>
-  <si>
-    <t>Kirkland Vitamina C Masticable 500 mg (500 tabletas)</t>
-  </si>
-  <si>
-    <t>VM-VITC-500</t>
-  </si>
-  <si>
-    <t>Nature's Bounty Hair, Skin &amp; Nails (250 softgels)</t>
-  </si>
-  <si>
-    <t>CP-HSN-250</t>
+    <t>Nature's Truth Vinagre de Manzana Orgánico 500 mg (120 gomitas)</t>
+  </si>
+  <si>
+    <t>Nature's Truth</t>
+  </si>
+  <si>
+    <t>SUP-ACV-120</t>
+  </si>
+  <si>
+    <t>Nutricost Selenio 200 mcg (240 cápsulas)</t>
+  </si>
+  <si>
+    <t>Nutricost</t>
+  </si>
+  <si>
+    <t>VM-SELENIO-240</t>
+  </si>
+  <si>
+    <t>Orgain Creatina Monohidratada Micronizada sin sabor (675 g)</t>
+  </si>
+  <si>
+    <t>Orgain</t>
+  </si>
+  <si>
+    <t>SUP-CREATINA-675</t>
+  </si>
+  <si>
+    <t>trunature Probiótico Digestivo Avanzado (100 cápsulas)</t>
+  </si>
+  <si>
+    <t>trunature</t>
+  </si>
+  <si>
+    <t>SUP-PROBIO-100</t>
+  </si>
+  <si>
+    <t>trunature Resveratrol Plus (140 cápsulas)</t>
+  </si>
+  <si>
+    <t>SUP-RESV-140</t>
+  </si>
+  <si>
+    <t>Vitamina E 1000 UI para salud del corazón (60 cápsulas)</t>
+  </si>
+  <si>
+    <t>VM-VITE1000-60</t>
+  </si>
+  <si>
+    <t>youtheory Ashwagandha (180 gomitas, frutos rojos)</t>
+  </si>
+  <si>
+    <t>youtheory</t>
+  </si>
+  <si>
+    <t>SUP-ASHGUM-180</t>
+  </si>
+  <si>
+    <t>youtheory Ashwagandha 1000 mg (180 cápsulas)</t>
+  </si>
+  <si>
+    <t>SUP-ASH-180</t>
+  </si>
+  <si>
+    <t>youtheory Colágeno Verisol con Biotina (345 comprimidos)</t>
+  </si>
+  <si>
+    <t>SUP-COLLVER-345</t>
   </si>
   <si>
     <t>youtheory Daily Fat Burner (130 cápsulas)</t>
   </si>
   <si>
-    <t>youtheory</t>
-  </si>
-  <si>
-    <t>Suplementos</t>
-  </si>
-  <si>
     <t>SUP-FATBURN-130</t>
   </si>
   <si>
-    <t>youtheory Ashwagandha (180 gomitas, frutos rojos)</t>
-  </si>
-  <si>
-    <t>SUP-ASHGUM-180</t>
-  </si>
-  <si>
-    <t>youtheory Ashwagandha 1000 mg (180 cápsulas)</t>
-  </si>
-  <si>
-    <t>SUP-ASH-180</t>
-  </si>
-  <si>
-    <t>youtheory Colágeno Verisol con Biotina (345 comprimidos)</t>
-  </si>
-  <si>
-    <t>SUP-COLLVER-345</t>
-  </si>
-  <si>
-    <t>Nature Made Magnesio Glicinato 100 mg (90 gomitas)</t>
-  </si>
-  <si>
-    <t>VM-MAGGUM-90</t>
-  </si>
-  <si>
-    <t>Nature Made Prenatal Ácido Fólico + DHA (150 softgels)</t>
-  </si>
-  <si>
-    <t>VM-PRENATAL-150</t>
-  </si>
-  <si>
-    <t>Kirkland Omega-3 Aceite de Pescado 1000 mg (400 softgels)</t>
-  </si>
-  <si>
-    <t>SUP-FISHOIL-400</t>
-  </si>
-  <si>
-    <t>Kirkland Vitamina E 180 mg (500 softgels)</t>
-  </si>
-  <si>
-    <t>VM-VITE-500</t>
-  </si>
-  <si>
-    <t>Kirkland Calcio 600 mg con Vitamina D3 (500 tabletas)</t>
-  </si>
-  <si>
-    <t>VM-CALCIO-500</t>
-  </si>
-  <si>
-    <t>Force Factor Ultra Berberina 1200 mg (60 cápsulas)</t>
-  </si>
-  <si>
-    <t>Force Factor</t>
-  </si>
-  <si>
-    <t>SUP-BERBER-60</t>
-  </si>
-  <si>
-    <t>Vitamina E 1000 UI para salud del corazón (60 cápsulas)</t>
-  </si>
-  <si>
-    <t>VM-VITE1000-60</t>
-  </si>
-  <si>
-    <t>trunature Resveratrol Plus (140 cápsulas)</t>
-  </si>
-  <si>
-    <t>trunature</t>
-  </si>
-  <si>
-    <t>SUP-RESV-140</t>
-  </si>
-  <si>
-    <t>Nature's Truth Vinagre de Manzana Orgánico 500 mg (120 gomitas)</t>
-  </si>
-  <si>
-    <t>Nature's Truth</t>
-  </si>
-  <si>
-    <t>SUP-ACV-120</t>
-  </si>
-  <si>
-    <t>Kirkland B-12 5000 mcg Disolución Rápida (300 tabletas)</t>
-  </si>
-  <si>
-    <t>VM-B12-300</t>
-  </si>
-  <si>
-    <t>Natrol Melatonina 5 mg Disolución Rápida (250 tabletas)</t>
-  </si>
-  <si>
-    <t>Natrol</t>
-  </si>
-  <si>
-    <t>SUP-MELA-250</t>
-  </si>
-  <si>
-    <t>trunature Probiótico Digestivo Avanzado (100 cápsulas)</t>
-  </si>
-  <si>
-    <t>SUP-PROBIO-100</t>
-  </si>
-  <si>
-    <t>Carlyle Panax Ginseng + Ginkgo Biloba 5.000 mg (120 cápsulas)</t>
-  </si>
-  <si>
-    <t>Carlyle</t>
-  </si>
-  <si>
-    <t>SUP-GINSENG-120</t>
-  </si>
-  <si>
-    <t>Nature Made Vitamina D3 25 mcg (650 softgels)</t>
-  </si>
-  <si>
-    <t>VM-VITD3-650</t>
-  </si>
-  <si>
-    <t>Nutricost Selenio 200 mcg (240 cápsulas)</t>
-  </si>
-  <si>
-    <t>Nutricost</t>
-  </si>
-  <si>
-    <t>VM-SELENIO-240</t>
-  </si>
-  <si>
-    <t>Kirkland Minoxidil 5% para hombres (tubo 60 mL)</t>
-  </si>
-  <si>
-    <t>CP-MINOXIDIL</t>
-  </si>
-  <si>
-    <t>Kirkland Glucosamina y Condroitina (280 tabletas)</t>
-  </si>
-  <si>
-    <t>SUP-GLUCO-280</t>
-  </si>
-  <si>
-    <t>Nature Made CoQ10 200 mg (140 softgels)</t>
-  </si>
-  <si>
-    <t>SUP-COQ10-140</t>
-  </si>
-  <si>
-    <t>Orgain Creatina Monohidratada Micronizada sin sabor (675 g)</t>
-  </si>
-  <si>
-    <t>Orgain</t>
-  </si>
-  <si>
-    <t>SUP-CREATINA-675</t>
-  </si>
-  <si>
-    <t>Feel Good Berberina Fitosoma de alta absorción (120 cápsulas veganas)</t>
-  </si>
-  <si>
-    <t>Feel Good Company</t>
-  </si>
-  <si>
-    <t>SUP-BERBER-FG120</t>
-  </si>
-  <si>
     <t>RESUMEN DEL INVENTARIO</t>
   </si>
   <si>
@@ -306,7 +306,7 @@
     <t>Se recalcula solo cuando cambias las cantidades en la hoja Inventario.</t>
   </si>
   <si>
-    <t>Generado: 29/10/2026, 9:40:56 a. m.</t>
+    <t>Generado: 29/10/2026, 9:44:02 a. m.</t>
   </si>
   <si>
     <t>CÓMO USAR ESTE EXCEL</t>
@@ -1008,10 +1008,10 @@
         <v>12</v>
       </c>
       <c r="D5" s="7">
-        <v>170000</v>
+        <v>120000</v>
       </c>
       <c r="E5" s="8">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F5" s="9" t="s">
         <v>13</v>
@@ -1034,7 +1034,7 @@
         <v>12</v>
       </c>
       <c r="D6" s="7">
-        <v>130000</v>
+        <v>160000</v>
       </c>
       <c r="E6" s="8">
         <v>2</v>
@@ -1054,16 +1054,16 @@
         <v>18</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="C7" s="6" t="s">
-        <v>19</v>
+        <v>12</v>
       </c>
       <c r="D7" s="7">
-        <v>130000</v>
+        <v>120000</v>
       </c>
       <c r="E7" s="8">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F7" s="9" t="s">
         <v>13</v>
@@ -1083,7 +1083,7 @@
         <v>22</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>12</v>
+        <v>23</v>
       </c>
       <c r="D8" s="7">
         <v>130000</v>
@@ -1098,24 +1098,24 @@
         <f>IF(F8="NO","Oculto",IF(E8&lt;=0,"AGOTADO",IF(E8&lt;=5,"Últimas unidades","Disponible")))</f>
       </c>
       <c r="H8" s="11" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="9" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A9" s="5" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B9" s="6" t="s">
-        <v>11</v>
+        <v>22</v>
       </c>
       <c r="C9" s="6" t="s">
-        <v>12</v>
+        <v>23</v>
       </c>
       <c r="D9" s="7">
-        <v>160000</v>
+        <v>110000</v>
       </c>
       <c r="E9" s="8">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F9" s="9" t="s">
         <v>13</v>
@@ -1124,12 +1124,12 @@
         <f>IF(F9="NO","Oculto",IF(E9&lt;=0,"AGOTADO",IF(E9&lt;=5,"Últimas unidades","Disponible")))</f>
       </c>
       <c r="H9" s="11" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
     </row>
     <row r="10" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A10" s="12" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B10" s="4" t="s">
         <v>22</v>
@@ -1138,7 +1138,7 @@
         <v>12</v>
       </c>
       <c r="D10" s="7">
-        <v>130000</v>
+        <v>160000</v>
       </c>
       <c r="E10" s="8">
         <v>1</v>
@@ -1150,24 +1150,24 @@
         <f>IF(F10="NO","Oculto",IF(E10&lt;=0,"AGOTADO",IF(E10&lt;=5,"Últimas unidades","Disponible")))</f>
       </c>
       <c r="H10" s="11" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
     <row r="11" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A11" s="5" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="B11" s="6" t="s">
-        <v>16</v>
+        <v>22</v>
       </c>
       <c r="C11" s="6" t="s">
-        <v>19</v>
+        <v>30</v>
       </c>
       <c r="D11" s="7">
-        <v>120000</v>
+        <v>60000</v>
       </c>
       <c r="E11" s="8">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="F11" s="9" t="s">
         <v>13</v>
@@ -1176,21 +1176,21 @@
         <f>IF(F11="NO","Oculto",IF(E11&lt;=0,"AGOTADO",IF(E11&lt;=5,"Últimas unidades","Disponible")))</f>
       </c>
       <c r="H11" s="11" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
     </row>
     <row r="12" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A12" s="12" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>31</v>
+        <v>22</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>32</v>
+        <v>12</v>
       </c>
       <c r="D12" s="7">
-        <v>160000</v>
+        <v>130000</v>
       </c>
       <c r="E12" s="8">
         <v>0</v>
@@ -1210,16 +1210,16 @@
         <v>34</v>
       </c>
       <c r="B13" s="6" t="s">
-        <v>31</v>
+        <v>22</v>
       </c>
       <c r="C13" s="6" t="s">
-        <v>32</v>
+        <v>23</v>
       </c>
       <c r="D13" s="7">
-        <v>160000</v>
+        <v>130000</v>
       </c>
       <c r="E13" s="8">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F13" s="9" t="s">
         <v>13</v>
@@ -1236,16 +1236,16 @@
         <v>36</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>31</v>
+        <v>22</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>32</v>
+        <v>23</v>
       </c>
       <c r="D14" s="7">
-        <v>160000</v>
+        <v>130000</v>
       </c>
       <c r="E14" s="8">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F14" s="9" t="s">
         <v>13</v>
@@ -1262,16 +1262,16 @@
         <v>38</v>
       </c>
       <c r="B15" s="6" t="s">
-        <v>31</v>
+        <v>22</v>
       </c>
       <c r="C15" s="6" t="s">
-        <v>32</v>
+        <v>23</v>
       </c>
       <c r="D15" s="7">
-        <v>200000</v>
+        <v>120000</v>
       </c>
       <c r="E15" s="8">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="F15" s="9" t="s">
         <v>13</v>
@@ -1288,16 +1288,16 @@
         <v>40</v>
       </c>
       <c r="B16" s="4" t="s">
-        <v>11</v>
+        <v>41</v>
       </c>
       <c r="C16" s="4" t="s">
         <v>12</v>
       </c>
       <c r="D16" s="7">
-        <v>130000</v>
+        <v>140000</v>
       </c>
       <c r="E16" s="8">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="F16" s="9" t="s">
         <v>13</v>
@@ -1306,21 +1306,21 @@
         <f>IF(F16="NO","Oculto",IF(E16&lt;=0,"AGOTADO",IF(E16&lt;=5,"Últimas unidades","Disponible")))</f>
       </c>
       <c r="H16" s="11" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
     </row>
     <row r="17" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A17" s="5" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B17" s="6" t="s">
-        <v>11</v>
+        <v>44</v>
       </c>
       <c r="C17" s="6" t="s">
         <v>12</v>
       </c>
       <c r="D17" s="7">
-        <v>200000</v>
+        <v>260000</v>
       </c>
       <c r="E17" s="8">
         <v>1</v>
@@ -1332,24 +1332,24 @@
         <f>IF(F17="NO","Oculto",IF(E17&lt;=0,"AGOTADO",IF(E17&lt;=5,"Últimas unidades","Disponible")))</f>
       </c>
       <c r="H17" s="11" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
     </row>
     <row r="18" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A18" s="12" t="s">
+        <v>46</v>
+      </c>
+      <c r="B18" s="4" t="s">
         <v>44</v>
       </c>
-      <c r="B18" s="4" t="s">
-        <v>22</v>
-      </c>
       <c r="C18" s="4" t="s">
-        <v>32</v>
+        <v>23</v>
       </c>
       <c r="D18" s="7">
-        <v>130000</v>
+        <v>170000</v>
       </c>
       <c r="E18" s="8">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F18" s="9" t="s">
         <v>13</v>
@@ -1358,24 +1358,24 @@
         <f>IF(F18="NO","Oculto",IF(E18&lt;=0,"AGOTADO",IF(E18&lt;=5,"Últimas unidades","Disponible")))</f>
       </c>
       <c r="H18" s="11" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
     </row>
     <row r="19" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A19" s="5" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="B19" s="6" t="s">
-        <v>22</v>
+        <v>44</v>
       </c>
       <c r="C19" s="6" t="s">
-        <v>12</v>
+        <v>23</v>
       </c>
       <c r="D19" s="7">
-        <v>120000</v>
+        <v>130000</v>
       </c>
       <c r="E19" s="8">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="F19" s="9" t="s">
         <v>13</v>
@@ -1384,24 +1384,24 @@
         <f>IF(F19="NO","Oculto",IF(E19&lt;=0,"AGOTADO",IF(E19&lt;=5,"Últimas unidades","Disponible")))</f>
       </c>
       <c r="H19" s="11" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
     </row>
     <row r="20" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A20" s="12" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="B20" s="4" t="s">
-        <v>22</v>
+        <v>44</v>
       </c>
       <c r="C20" s="4" t="s">
-        <v>12</v>
+        <v>23</v>
       </c>
       <c r="D20" s="7">
-        <v>110000</v>
+        <v>200000</v>
       </c>
       <c r="E20" s="8">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F20" s="9" t="s">
         <v>13</v>
@@ -1410,21 +1410,21 @@
         <f>IF(F20="NO","Oculto",IF(E20&lt;=0,"AGOTADO",IF(E20&lt;=5,"Últimas unidades","Disponible")))</f>
       </c>
       <c r="H20" s="11" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
     </row>
     <row r="21" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A21" s="5" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="B21" s="6" t="s">
-        <v>51</v>
+        <v>44</v>
       </c>
       <c r="C21" s="6" t="s">
-        <v>32</v>
+        <v>23</v>
       </c>
       <c r="D21" s="7">
-        <v>120000</v>
+        <v>160000</v>
       </c>
       <c r="E21" s="8">
         <v>0</v>
@@ -1436,24 +1436,24 @@
         <f>IF(F21="NO","Oculto",IF(E21&lt;=0,"AGOTADO",IF(E21&lt;=5,"Últimas unidades","Disponible")))</f>
       </c>
       <c r="H21" s="11" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
     </row>
     <row r="22" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A22" s="12" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="B22" s="4" t="s">
-        <v>16</v>
+        <v>44</v>
       </c>
       <c r="C22" s="4" t="s">
-        <v>12</v>
+        <v>23</v>
       </c>
       <c r="D22" s="7">
-        <v>120000</v>
+        <v>140000</v>
       </c>
       <c r="E22" s="8">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F22" s="9" t="s">
         <v>13</v>
@@ -1462,21 +1462,21 @@
         <f>IF(F22="NO","Oculto",IF(E22&lt;=0,"AGOTADO",IF(E22&lt;=5,"Últimas unidades","Disponible")))</f>
       </c>
       <c r="H22" s="11" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
     </row>
     <row r="23" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A23" s="5" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="B23" s="6" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="C23" s="6" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="D23" s="7">
-        <v>140000</v>
+        <v>120000</v>
       </c>
       <c r="E23" s="8">
         <v>2</v>
@@ -1488,18 +1488,18 @@
         <f>IF(F23="NO","Oculto",IF(E23&lt;=0,"AGOTADO",IF(E23&lt;=5,"Últimas unidades","Disponible")))</f>
       </c>
       <c r="H23" s="11" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
     </row>
     <row r="24" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A24" s="12" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="B24" s="4" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="C24" s="4" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="D24" s="7">
         <v>130000</v>
@@ -1522,16 +1522,16 @@
         <v>61</v>
       </c>
       <c r="B25" s="6" t="s">
-        <v>22</v>
+        <v>57</v>
       </c>
       <c r="C25" s="6" t="s">
-        <v>12</v>
+        <v>23</v>
       </c>
       <c r="D25" s="7">
         <v>130000</v>
       </c>
       <c r="E25" s="8">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F25" s="9" t="s">
         <v>13</v>
@@ -1551,13 +1551,13 @@
         <v>64</v>
       </c>
       <c r="C26" s="4" t="s">
-        <v>32</v>
+        <v>12</v>
       </c>
       <c r="D26" s="7">
-        <v>140000</v>
+        <v>130000</v>
       </c>
       <c r="E26" s="8">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F26" s="9" t="s">
         <v>13</v>
@@ -1574,16 +1574,16 @@
         <v>66</v>
       </c>
       <c r="B27" s="6" t="s">
-        <v>56</v>
+        <v>67</v>
       </c>
       <c r="C27" s="6" t="s">
-        <v>32</v>
+        <v>23</v>
       </c>
       <c r="D27" s="7">
-        <v>130000</v>
+        <v>160000</v>
       </c>
       <c r="E27" s="8">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F27" s="9" t="s">
         <v>13</v>
@@ -1592,24 +1592,24 @@
         <f>IF(F27="NO","Oculto",IF(E27&lt;=0,"AGOTADO",IF(E27&lt;=5,"Últimas unidades","Disponible")))</f>
       </c>
       <c r="H27" s="11" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
     </row>
     <row r="28" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A28" s="12" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="B28" s="4" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="C28" s="4" t="s">
-        <v>32</v>
+        <v>12</v>
       </c>
       <c r="D28" s="7">
-        <v>120000</v>
+        <v>160000</v>
       </c>
       <c r="E28" s="8">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F28" s="9" t="s">
         <v>13</v>
@@ -1618,21 +1618,21 @@
         <f>IF(F28="NO","Oculto",IF(E28&lt;=0,"AGOTADO",IF(E28&lt;=5,"Últimas unidades","Disponible")))</f>
       </c>
       <c r="H28" s="11" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
     </row>
     <row r="29" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A29" s="5" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="B29" s="6" t="s">
-        <v>11</v>
+        <v>73</v>
       </c>
       <c r="C29" s="6" t="s">
         <v>12</v>
       </c>
       <c r="D29" s="7">
-        <v>140000</v>
+        <v>130000</v>
       </c>
       <c r="E29" s="8">
         <v>1</v>
@@ -1644,21 +1644,21 @@
         <f>IF(F29="NO","Oculto",IF(E29&lt;=0,"AGOTADO",IF(E29&lt;=5,"Últimas unidades","Disponible")))</f>
       </c>
       <c r="H29" s="11" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
     </row>
     <row r="30" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A30" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="B30" s="4" t="s">
         <v>73</v>
-      </c>
-      <c r="B30" s="4" t="s">
-        <v>74</v>
       </c>
       <c r="C30" s="4" t="s">
         <v>12</v>
       </c>
       <c r="D30" s="7">
-        <v>160000</v>
+        <v>140000</v>
       </c>
       <c r="E30" s="8">
         <v>2</v>
@@ -1670,24 +1670,24 @@
         <f>IF(F30="NO","Oculto",IF(E30&lt;=0,"AGOTADO",IF(E30&lt;=5,"Últimas unidades","Disponible")))</f>
       </c>
       <c r="H30" s="11" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
     </row>
     <row r="31" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A31" s="5" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="B31" s="6" t="s">
-        <v>22</v>
+        <v>57</v>
       </c>
       <c r="C31" s="6" t="s">
-        <v>19</v>
+        <v>23</v>
       </c>
       <c r="D31" s="7">
-        <v>60000</v>
+        <v>120000</v>
       </c>
       <c r="E31" s="8">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="F31" s="9" t="s">
         <v>13</v>
@@ -1696,24 +1696,24 @@
         <f>IF(F31="NO","Oculto",IF(E31&lt;=0,"AGOTADO",IF(E31&lt;=5,"Últimas unidades","Disponible")))</f>
       </c>
       <c r="H31" s="11" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
     </row>
     <row r="32" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A32" s="12" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="B32" s="4" t="s">
-        <v>22</v>
+        <v>80</v>
       </c>
       <c r="C32" s="4" t="s">
-        <v>32</v>
+        <v>12</v>
       </c>
       <c r="D32" s="7">
         <v>160000</v>
       </c>
       <c r="E32" s="8">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F32" s="9" t="s">
         <v>13</v>
@@ -1722,24 +1722,24 @@
         <f>IF(F32="NO","Oculto",IF(E32&lt;=0,"AGOTADO",IF(E32&lt;=5,"Últimas unidades","Disponible")))</f>
       </c>
       <c r="H32" s="11" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
     </row>
     <row r="33" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A33" s="5" t="s">
+        <v>82</v>
+      </c>
+      <c r="B33" s="6" t="s">
         <v>80</v>
       </c>
-      <c r="B33" s="6" t="s">
-        <v>11</v>
-      </c>
       <c r="C33" s="6" t="s">
-        <v>32</v>
+        <v>12</v>
       </c>
       <c r="D33" s="7">
-        <v>260000</v>
+        <v>160000</v>
       </c>
       <c r="E33" s="8">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F33" s="9" t="s">
         <v>13</v>
@@ -1748,24 +1748,24 @@
         <f>IF(F33="NO","Oculto",IF(E33&lt;=0,"AGOTADO",IF(E33&lt;=5,"Últimas unidades","Disponible")))</f>
       </c>
       <c r="H33" s="11" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
     </row>
     <row r="34" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A34" s="12" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="B34" s="4" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="C34" s="4" t="s">
-        <v>32</v>
+        <v>12</v>
       </c>
       <c r="D34" s="7">
-        <v>160000</v>
+        <v>200000</v>
       </c>
       <c r="E34" s="8">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F34" s="9" t="s">
         <v>13</v>
@@ -1774,24 +1774,24 @@
         <f>IF(F34="NO","Oculto",IF(E34&lt;=0,"AGOTADO",IF(E34&lt;=5,"Últimas unidades","Disponible")))</f>
       </c>
       <c r="H34" s="11" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
     </row>
     <row r="35" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A35" s="5" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="B35" s="6" t="s">
-        <v>86</v>
+        <v>80</v>
       </c>
       <c r="C35" s="6" t="s">
-        <v>32</v>
+        <v>12</v>
       </c>
       <c r="D35" s="7">
         <v>160000</v>
       </c>
       <c r="E35" s="8">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F35" s="9" t="s">
         <v>13</v>

</xml_diff>